<commit_message>
Switch STR comparison to H1 (Jan-Jun) of each year, 2026 included
- Overview and report change view now compare H1 2023/2024/2025/2026
- H1 2026 uses STR's official YTD row; prior years day-weighted from monthly
- Bottom tables show H1 averages by year

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GzrfbzxdPZVRCw2bYpGG1J
</commit_message>
<xml_diff>
--- a/output/STR_Bangkok_by_segment_2023-2026.xlsx
+++ b/output/STR_Bangkok_by_segment_2023-2026.xlsx
@@ -238,7 +238,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Occupancy (%) — yearly average</a:t>
+              <a:t>Occupancy (%) — H1 average by year</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -273,12 +273,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$5:$D$5</f>
+              <f>'Overview'!$B$5:$E$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$5:$D$5</f>
+              <f>'Overview'!$B$5:$E$5</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -309,12 +309,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$5:$D$5</f>
+              <f>'Overview'!$B$5:$E$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$6:$D$6</f>
+              <f>'Overview'!$B$6:$E$6</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -345,12 +345,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$5:$D$5</f>
+              <f>'Overview'!$B$5:$E$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$7:$D$7</f>
+              <f>'Overview'!$B$7:$E$7</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -381,12 +381,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$5:$D$5</f>
+              <f>'Overview'!$B$5:$E$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$8:$D$8</f>
+              <f>'Overview'!$B$8:$E$8</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -414,12 +414,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$5:$D$5</f>
+              <f>'Overview'!$B$5:$E$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$9:$D$9</f>
+              <f>'Overview'!$B$9:$E$9</f>
             </numRef>
           </val>
         </ser>
@@ -472,7 +472,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>ADR (THB) — yearly average</a:t>
+              <a:t>ADR (THB) — H1 average by year</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -507,12 +507,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$21:$D$21</f>
+              <f>'Overview'!$B$21:$E$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$21:$D$21</f>
+              <f>'Overview'!$B$21:$E$21</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$21:$D$21</f>
+              <f>'Overview'!$B$21:$E$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$22:$D$22</f>
+              <f>'Overview'!$B$22:$E$22</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -579,12 +579,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$21:$D$21</f>
+              <f>'Overview'!$B$21:$E$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$23:$D$23</f>
+              <f>'Overview'!$B$23:$E$23</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -615,12 +615,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$21:$D$21</f>
+              <f>'Overview'!$B$21:$E$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$24:$D$24</f>
+              <f>'Overview'!$B$24:$E$24</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -648,12 +648,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$21:$D$21</f>
+              <f>'Overview'!$B$21:$E$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$25:$D$25</f>
+              <f>'Overview'!$B$25:$E$25</f>
             </numRef>
           </val>
         </ser>
@@ -706,7 +706,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>RevPAR (THB) — yearly average</a:t>
+              <a:t>RevPAR (THB) — H1 average by year</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -741,12 +741,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$37:$D$37</f>
+              <f>'Overview'!$B$37:$E$37</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$37:$D$37</f>
+              <f>'Overview'!$B$37:$E$37</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -777,12 +777,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$37:$D$37</f>
+              <f>'Overview'!$B$37:$E$37</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$38:$D$38</f>
+              <f>'Overview'!$B$38:$E$38</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$37:$D$37</f>
+              <f>'Overview'!$B$37:$E$37</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$39:$D$39</f>
+              <f>'Overview'!$B$39:$E$39</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -849,12 +849,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$37:$D$37</f>
+              <f>'Overview'!$B$37:$E$37</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$40:$D$40</f>
+              <f>'Overview'!$B$40:$E$40</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -882,12 +882,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Overview'!$B$37:$D$37</f>
+              <f>'Overview'!$B$37:$E$37</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$41:$D$41</f>
+              <f>'Overview'!$B$41:$E$41</f>
             </numRef>
           </val>
         </ser>
@@ -1631,7 +1631,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>10</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -1653,7 +1653,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>10</col>
       <colOff>0</colOff>
       <row>19</row>
       <rowOff>0</rowOff>
@@ -1675,7 +1675,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>10</col>
       <colOff>0</colOff>
       <row>35</row>
       <rowOff>0</rowOff>
@@ -2068,7 +2068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2078,19 +2078,21 @@
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bangkok STR — market class comparison: change 2023–2025</t>
+          <t>Bangkok STR — market class comparison: H1 (Jan–Jun) of each year</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Yearly averages by market class (STR 'Total' rows) with % change. Occupancy = %, ADR &amp; RevPAR = THB. '24 vs 23' / '25 vs 24' are STR's own % Chg.</t>
+          <t>First-half (Jan–Jun) averages by market class, 2023–2026, with % change. Occupancy = %, ADR &amp; RevPAR = THB. H1 2023–2025 are day-weighted from STR monthly data; H1 2026 is STR's own YTD row.</t>
         </is>
       </c>
     </row>
@@ -2109,32 +2111,42 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>H1 2023</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>H1 2024</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>H1 2025</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
+          <t>H1 2026</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
           <t>24 vs 23</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>25 vs 24</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>25 vs 23</t>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>26 vs 25</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>26 vs 23</t>
         </is>
       </c>
     </row>
@@ -2145,22 +2157,28 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>68.7</v>
+        <v>67.2</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>73.40000000000001</v>
+        <v>72.7</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>67</v>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>6.9</v>
-      </c>
-      <c r="F6" s="9" t="n">
-        <v>-8.699999999999999</v>
+        <v>65.09999999999999</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>8.1</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>-2.5</v>
+        <v>-10.5</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>-0.1</v>
       </c>
     </row>
     <row r="7">
@@ -2170,22 +2188,28 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>72.2</v>
+        <v>71</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>75.8</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>69.59999999999999</v>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="F7" s="9" t="n">
-        <v>-8.1</v>
+        <v>68.59999999999999</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>7.8</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>-3.5</v>
+        <v>-10.4</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>-2.9</v>
       </c>
     </row>
     <row r="8">
@@ -2195,22 +2219,28 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>71.3</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>77</v>
+        <v>75.8</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>74.2</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="F8" s="9" t="n">
-        <v>-3.6</v>
-      </c>
-      <c r="G8" s="8" t="n">
-        <v>3.9</v>
+        <v>71.8</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>75.40000000000001</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -2220,22 +2250,28 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>71.7</v>
+        <v>70.3</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>76.3</v>
+        <v>74.3</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>75.90000000000001</v>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="F9" s="9" t="n">
-        <v>-0.6</v>
+        <v>74.3</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>76.8</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>5.6</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>5.8</v>
+        <v>0</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -2253,32 +2289,42 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>H1 2023</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>H1 2024</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>H1 2025</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
+          <t>H1 2026</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
           <t>24 vs 23</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>25 vs 24</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>25 vs 23</t>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>26 vs 25</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>26 vs 23</t>
         </is>
       </c>
     </row>
@@ -2289,22 +2335,28 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>6685</v>
+        <v>6620</v>
       </c>
       <c r="C22" s="13" t="n">
-        <v>6984</v>
+        <v>6858</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>6998</v>
-      </c>
-      <c r="E22" s="8" t="n">
-        <v>4.5</v>
+        <v>7007</v>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>6845</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>0.2</v>
+        <v>3.6</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>4.7</v>
+        <v>2.2</v>
+      </c>
+      <c r="H22" s="9" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="I22" s="8" t="n">
+        <v>3.4</v>
       </c>
     </row>
     <row r="23">
@@ -2314,22 +2366,28 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>4258</v>
+        <v>4205</v>
       </c>
       <c r="C23" s="13" t="n">
-        <v>4492</v>
+        <v>4399</v>
       </c>
       <c r="D23" s="13" t="n">
-        <v>4391</v>
-      </c>
-      <c r="E23" s="8" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="F23" s="9" t="n">
-        <v>-2.2</v>
+        <v>4430</v>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>4301</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>4.6</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>3.1</v>
+        <v>0.7</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>-2.9</v>
+      </c>
+      <c r="I23" s="8" t="n">
+        <v>2.3</v>
       </c>
     </row>
     <row r="24">
@@ -2339,22 +2397,28 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>2906</v>
+        <v>2838</v>
       </c>
       <c r="C24" s="13" t="n">
-        <v>3148</v>
+        <v>3038</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>3099</v>
-      </c>
-      <c r="E24" s="8" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>-1.6</v>
+        <v>3130</v>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>2990</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>7</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>6.6</v>
+        <v>3.1</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="I24" s="8" t="n">
+        <v>5.4</v>
       </c>
     </row>
     <row r="25">
@@ -2364,22 +2428,28 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>2548</v>
+        <v>2431</v>
       </c>
       <c r="C25" s="13" t="n">
-        <v>2831</v>
+        <v>2697</v>
       </c>
       <c r="D25" s="13" t="n">
-        <v>2813</v>
-      </c>
-      <c r="E25" s="8" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="F25" s="9" t="n">
-        <v>-0.6</v>
+        <v>2834</v>
+      </c>
+      <c r="E25" s="13" t="n">
+        <v>2634</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>10.9</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>10.4</v>
+        <v>5.1</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>-7</v>
+      </c>
+      <c r="I25" s="8" t="n">
+        <v>8.4</v>
       </c>
     </row>
     <row r="36">
@@ -2397,32 +2467,42 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>H1 2023</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>H1 2024</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>H1 2025</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
+          <t>H1 2026</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
           <t>24 vs 23</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>25 vs 24</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>25 vs 23</t>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>26 vs 25</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>26 vs 23</t>
         </is>
       </c>
     </row>
@@ -2433,22 +2513,28 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>4593</v>
+        <v>4452</v>
       </c>
       <c r="C38" s="13" t="n">
-        <v>5129</v>
+        <v>4987</v>
       </c>
       <c r="D38" s="13" t="n">
-        <v>4691</v>
-      </c>
-      <c r="E38" s="8" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="F38" s="9" t="n">
-        <v>-8.5</v>
-      </c>
-      <c r="G38" s="8" t="n">
-        <v>2.1</v>
+        <v>4560</v>
+      </c>
+      <c r="E38" s="13" t="n">
+        <v>4600</v>
+      </c>
+      <c r="F38" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="G38" s="9" t="n">
+        <v>-8.6</v>
+      </c>
+      <c r="H38" s="8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I38" s="8" t="n">
+        <v>3.3</v>
       </c>
     </row>
     <row r="39">
@@ -2458,22 +2544,28 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>3073</v>
+        <v>2987</v>
       </c>
       <c r="C39" s="13" t="n">
-        <v>3405</v>
+        <v>3369</v>
       </c>
       <c r="D39" s="13" t="n">
-        <v>3057</v>
-      </c>
-      <c r="E39" s="8" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="F39" s="9" t="n">
-        <v>-10.2</v>
+        <v>3039</v>
+      </c>
+      <c r="E39" s="13" t="n">
+        <v>2965</v>
+      </c>
+      <c r="F39" s="8" t="n">
+        <v>12.8</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>-0.5</v>
+        <v>-9.800000000000001</v>
+      </c>
+      <c r="H39" s="9" t="n">
+        <v>-2.4</v>
+      </c>
+      <c r="I39" s="9" t="n">
+        <v>-0.7</v>
       </c>
     </row>
     <row r="40">
@@ -2483,22 +2575,28 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>2073</v>
+        <v>1975</v>
       </c>
       <c r="C40" s="13" t="n">
-        <v>2423</v>
+        <v>2301</v>
       </c>
       <c r="D40" s="13" t="n">
-        <v>2298</v>
-      </c>
-      <c r="E40" s="8" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="F40" s="9" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="G40" s="8" t="n">
-        <v>10.8</v>
+        <v>2247</v>
+      </c>
+      <c r="E40" s="13" t="n">
+        <v>2255</v>
+      </c>
+      <c r="F40" s="8" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="G40" s="9" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="H40" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I40" s="8" t="n">
+        <v>14.2</v>
       </c>
     </row>
     <row r="41">
@@ -2508,22 +2606,28 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1827</v>
+        <v>1710</v>
       </c>
       <c r="C41" s="13" t="n">
-        <v>2161</v>
+        <v>2003</v>
       </c>
       <c r="D41" s="13" t="n">
-        <v>2135</v>
-      </c>
-      <c r="E41" s="8" t="n">
-        <v>18.3</v>
-      </c>
-      <c r="F41" s="9" t="n">
-        <v>-1.2</v>
+        <v>2106</v>
+      </c>
+      <c r="E41" s="13" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F41" s="8" t="n">
+        <v>17.2</v>
       </c>
       <c r="G41" s="8" t="n">
-        <v>16.8</v>
+        <v>5.1</v>
+      </c>
+      <c r="H41" s="9" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="I41" s="8" t="n">
+        <v>18.4</v>
       </c>
     </row>
     <row r="52">

</xml_diff>

<commit_message>
Calculate all STR YTD figures from raw monthly data (Mae's decision)
- Every H1/YTD figure incl 2026 is day-weighted from monthly rows;
  STR's pre-computed YTD rows are no longer used anywhere
- Bangkok overall shows no vs-2025 change (no 2025 monthly data)
- Decision logged in docs/decisions/2026-08-03-str-ytd-calculate-ourselves.md

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GzrfbzxdPZVRCw2bYpGG1J
</commit_message>
<xml_diff>
--- a/output/STR_Bangkok_by_segment_2023-2026.xlsx
+++ b/output/STR_Bangkok_by_segment_2023-2026.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="+0.0&quot;%&quot;;-0.0&quot;%&quot;;0.0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,6 +78,9 @@
       <color rgb="00595959"/>
     </font>
     <font>
+      <color rgb="00808080"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="13"/>
@@ -122,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -148,7 +151,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2092,7 +2098,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>First-half (Jan–Jun) averages by market class, 2023–2026, with % change. Occupancy = %, ADR &amp; RevPAR = THB. H1 2023–2025 are day-weighted from STR monthly data; H1 2026 is STR's own YTD row.</t>
+          <t>First-half (Jan–Jun) averages by market class, 2023–2026, with % change. Occupancy = %, ADR &amp; RevPAR = THB. ALL years calculated from STR monthly data (Occ/RevPAR day-weighted, ADR room-night-weighted) — STR's own YTD rows are not used (Mae's decision, 2026-08-03).</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2172,7 @@
         <v>65.09999999999999</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>67.2</v>
+        <v>66.8</v>
       </c>
       <c r="F6" s="8" t="n">
         <v>8.1</v>
@@ -2175,10 +2181,10 @@
         <v>-10.5</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>3.3</v>
+        <v>2.6</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>-0.1</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="7">
@@ -2237,10 +2243,10 @@
         <v>-5.2</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>8.300000000000001</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="9">
@@ -2271,7 +2277,7 @@
         <v>3.4</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -2344,7 +2350,7 @@
         <v>7007</v>
       </c>
       <c r="E22" s="13" t="n">
-        <v>6845</v>
+        <v>7082</v>
       </c>
       <c r="F22" s="8" t="n">
         <v>3.6</v>
@@ -2352,11 +2358,11 @@
       <c r="G22" s="8" t="n">
         <v>2.2</v>
       </c>
-      <c r="H22" s="9" t="n">
-        <v>-2.3</v>
+      <c r="H22" s="8" t="n">
+        <v>1.1</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>3.4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23">
@@ -2406,7 +2412,7 @@
         <v>3130</v>
       </c>
       <c r="E24" s="13" t="n">
-        <v>2990</v>
+        <v>2991</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>7</v>
@@ -2437,7 +2443,7 @@
         <v>2834</v>
       </c>
       <c r="E25" s="13" t="n">
-        <v>2634</v>
+        <v>2635</v>
       </c>
       <c r="F25" s="8" t="n">
         <v>10.9</v>
@@ -2522,7 +2528,7 @@
         <v>4560</v>
       </c>
       <c r="E38" s="13" t="n">
-        <v>4600</v>
+        <v>4729</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>12</v>
@@ -2531,10 +2537,10 @@
         <v>-8.6</v>
       </c>
       <c r="H38" s="8" t="n">
-        <v>0.9</v>
+        <v>3.7</v>
       </c>
       <c r="I38" s="8" t="n">
-        <v>3.3</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="39">
@@ -2584,7 +2590,7 @@
         <v>2247</v>
       </c>
       <c r="E40" s="13" t="n">
-        <v>2255</v>
+        <v>2256</v>
       </c>
       <c r="F40" s="8" t="n">
         <v>16.5</v>
@@ -2593,7 +2599,7 @@
         <v>-2.3</v>
       </c>
       <c r="H40" s="8" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I40" s="8" t="n">
         <v>14.2</v>
@@ -2633,7 +2639,7 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>YTD 2026 (Jan–Jun) vs same period 2025</t>
+          <t>YTD 2026 (Jan–Jun) — calculated from monthly data, vs calculated H1 2025</t>
         </is>
       </c>
     </row>
@@ -2681,22 +2687,28 @@
         </is>
       </c>
       <c r="B54" s="7" t="n">
-        <v>71.7</v>
-      </c>
-      <c r="C54" s="8" t="n">
-        <v>3.9</v>
+        <v>70.5</v>
+      </c>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D54" s="13" t="n">
-        <v>3759</v>
-      </c>
-      <c r="E54" s="9" t="n">
-        <v>-5.3</v>
+        <v>3952</v>
+      </c>
+      <c r="E54" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>2694</v>
-      </c>
-      <c r="G54" s="9" t="n">
-        <v>-1.6</v>
+        <v>2787</v>
+      </c>
+      <c r="G54" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -2706,22 +2718,22 @@
         </is>
       </c>
       <c r="B55" s="7" t="n">
-        <v>67.2</v>
+        <v>66.8</v>
       </c>
       <c r="C55" s="8" t="n">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="D55" s="13" t="n">
-        <v>6845</v>
-      </c>
-      <c r="E55" s="9" t="n">
-        <v>-1.3</v>
+        <v>7082</v>
+      </c>
+      <c r="E55" s="8" t="n">
+        <v>1.1</v>
       </c>
       <c r="F55" s="13" t="n">
-        <v>4600</v>
+        <v>4729</v>
       </c>
       <c r="G55" s="8" t="n">
-        <v>1.7</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="56">
@@ -2734,19 +2746,19 @@
         <v>68.90000000000001</v>
       </c>
       <c r="C56" s="8" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="D56" s="13" t="n">
         <v>4301</v>
       </c>
       <c r="E56" s="9" t="n">
-        <v>-2.1</v>
+        <v>-2.9</v>
       </c>
       <c r="F56" s="13" t="n">
         <v>2965</v>
       </c>
       <c r="G56" s="9" t="n">
-        <v>-1.4</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="57">
@@ -2759,19 +2771,19 @@
         <v>75.40000000000001</v>
       </c>
       <c r="C57" s="8" t="n">
-        <v>4.7</v>
+        <v>5.1</v>
       </c>
       <c r="D57" s="13" t="n">
-        <v>2990</v>
+        <v>2991</v>
       </c>
       <c r="E57" s="9" t="n">
-        <v>-3.9</v>
+        <v>-4.5</v>
       </c>
       <c r="F57" s="13" t="n">
-        <v>2255</v>
+        <v>2256</v>
       </c>
       <c r="G57" s="8" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="58">
@@ -2784,19 +2796,19 @@
         <v>76.8</v>
       </c>
       <c r="C58" s="8" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="D58" s="13" t="n">
-        <v>2634</v>
+        <v>2635</v>
       </c>
       <c r="E58" s="9" t="n">
-        <v>-6.3</v>
+        <v>-7</v>
       </c>
       <c r="F58" s="13" t="n">
         <v>2024</v>
       </c>
       <c r="G58" s="9" t="n">
-        <v>-3.5</v>
+        <v>-3.9</v>
       </c>
     </row>
   </sheetData>
@@ -2822,7 +2834,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Bangkok STR — Occupancy by market class (monthly, This Year)</t>
         </is>
@@ -2863,7 +2875,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Jan 2023</t>
         </is>
@@ -2882,7 +2894,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Feb 2023</t>
         </is>
@@ -2901,7 +2913,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Mar 2023</t>
         </is>
@@ -2920,7 +2932,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Apr 2023</t>
         </is>
@@ -2939,7 +2951,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>May 2023</t>
         </is>
@@ -2958,7 +2970,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Jun 2023</t>
         </is>
@@ -2977,7 +2989,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Jul 2023</t>
         </is>
@@ -2996,7 +3008,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Aug 2023</t>
         </is>
@@ -3015,7 +3027,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Sep 2023</t>
         </is>
@@ -3034,7 +3046,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Oct 2023</t>
         </is>
@@ -3053,7 +3065,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Nov 2023</t>
         </is>
@@ -3072,7 +3084,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Dec 2023</t>
         </is>
@@ -3091,7 +3103,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Jan 2024</t>
         </is>
@@ -3110,7 +3122,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Feb 2024</t>
         </is>
@@ -3129,7 +3141,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Mar 2024</t>
         </is>
@@ -3148,7 +3160,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Apr 2024</t>
         </is>
@@ -3167,7 +3179,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>May 2024</t>
         </is>
@@ -3186,7 +3198,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Jun 2024</t>
         </is>
@@ -3205,7 +3217,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Jul 2024</t>
         </is>
@@ -3224,7 +3236,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Aug 2024</t>
         </is>
@@ -3243,7 +3255,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Sep 2024</t>
         </is>
@@ -3262,7 +3274,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Oct 2024</t>
         </is>
@@ -3281,7 +3293,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Nov 2024</t>
         </is>
@@ -3300,7 +3312,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
@@ -3319,7 +3331,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Jan 2025</t>
         </is>
@@ -3338,7 +3350,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>Feb 2025</t>
         </is>
@@ -3357,7 +3369,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>Mar 2025</t>
         </is>
@@ -3376,7 +3388,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Apr 2025</t>
         </is>
@@ -3395,7 +3407,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>May 2025</t>
         </is>
@@ -3414,7 +3426,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Jun 2025</t>
         </is>
@@ -3433,7 +3445,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="A35" s="17" t="inlineStr">
         <is>
           <t>Jul 2025</t>
         </is>
@@ -3452,7 +3464,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="inlineStr">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>Aug 2025</t>
         </is>
@@ -3471,7 +3483,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>Sep 2025</t>
         </is>
@@ -3490,7 +3502,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
@@ -3509,7 +3521,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>Nov 2025</t>
         </is>
@@ -3528,7 +3540,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>Dec 2025</t>
         </is>
@@ -3547,7 +3559,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>Jan 2026</t>
         </is>
@@ -3566,7 +3578,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="16" t="inlineStr">
+      <c r="A42" s="17" t="inlineStr">
         <is>
           <t>Feb 2026</t>
         </is>
@@ -3585,7 +3597,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
@@ -3604,7 +3616,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="16" t="inlineStr">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>Apr 2026</t>
         </is>
@@ -3623,7 +3635,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>May 2026</t>
         </is>
@@ -3642,7 +3654,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="16" t="inlineStr">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>Jun 2026</t>
         </is>
@@ -3683,7 +3695,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Bangkok STR — ADR by market class (monthly, This Year)</t>
         </is>
@@ -3724,7 +3736,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Jan 2023</t>
         </is>
@@ -3743,7 +3755,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Feb 2023</t>
         </is>
@@ -3762,7 +3774,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Mar 2023</t>
         </is>
@@ -3781,7 +3793,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Apr 2023</t>
         </is>
@@ -3800,7 +3812,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>May 2023</t>
         </is>
@@ -3819,7 +3831,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Jun 2023</t>
         </is>
@@ -3838,7 +3850,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Jul 2023</t>
         </is>
@@ -3857,7 +3869,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Aug 2023</t>
         </is>
@@ -3876,7 +3888,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Sep 2023</t>
         </is>
@@ -3895,7 +3907,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Oct 2023</t>
         </is>
@@ -3914,7 +3926,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Nov 2023</t>
         </is>
@@ -3933,7 +3945,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Dec 2023</t>
         </is>
@@ -3952,7 +3964,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Jan 2024</t>
         </is>
@@ -3971,7 +3983,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Feb 2024</t>
         </is>
@@ -3990,7 +4002,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Mar 2024</t>
         </is>
@@ -4009,7 +4021,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Apr 2024</t>
         </is>
@@ -4028,7 +4040,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>May 2024</t>
         </is>
@@ -4047,7 +4059,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Jun 2024</t>
         </is>
@@ -4066,7 +4078,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Jul 2024</t>
         </is>
@@ -4085,7 +4097,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Aug 2024</t>
         </is>
@@ -4104,7 +4116,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Sep 2024</t>
         </is>
@@ -4123,7 +4135,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Oct 2024</t>
         </is>
@@ -4142,7 +4154,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Nov 2024</t>
         </is>
@@ -4161,7 +4173,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
@@ -4180,7 +4192,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Jan 2025</t>
         </is>
@@ -4199,7 +4211,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>Feb 2025</t>
         </is>
@@ -4218,7 +4230,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>Mar 2025</t>
         </is>
@@ -4237,7 +4249,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Apr 2025</t>
         </is>
@@ -4256,7 +4268,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>May 2025</t>
         </is>
@@ -4275,7 +4287,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Jun 2025</t>
         </is>
@@ -4294,7 +4306,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="A35" s="17" t="inlineStr">
         <is>
           <t>Jul 2025</t>
         </is>
@@ -4313,7 +4325,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="inlineStr">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>Aug 2025</t>
         </is>
@@ -4332,7 +4344,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>Sep 2025</t>
         </is>
@@ -4351,7 +4363,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
@@ -4370,7 +4382,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>Nov 2025</t>
         </is>
@@ -4389,7 +4401,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>Dec 2025</t>
         </is>
@@ -4408,7 +4420,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>Jan 2026</t>
         </is>
@@ -4427,7 +4439,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="16" t="inlineStr">
+      <c r="A42" s="17" t="inlineStr">
         <is>
           <t>Feb 2026</t>
         </is>
@@ -4446,7 +4458,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
@@ -4465,7 +4477,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="16" t="inlineStr">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>Apr 2026</t>
         </is>
@@ -4484,7 +4496,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>May 2026</t>
         </is>
@@ -4503,7 +4515,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="16" t="inlineStr">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>Jun 2026</t>
         </is>
@@ -4544,7 +4556,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Bangkok STR — RevPAR by market class (monthly, This Year)</t>
         </is>
@@ -4585,7 +4597,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Jan 2023</t>
         </is>
@@ -4604,7 +4616,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Feb 2023</t>
         </is>
@@ -4623,7 +4635,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Mar 2023</t>
         </is>
@@ -4642,7 +4654,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Apr 2023</t>
         </is>
@@ -4661,7 +4673,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>May 2023</t>
         </is>
@@ -4680,7 +4692,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Jun 2023</t>
         </is>
@@ -4699,7 +4711,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Jul 2023</t>
         </is>
@@ -4718,7 +4730,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Aug 2023</t>
         </is>
@@ -4737,7 +4749,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Sep 2023</t>
         </is>
@@ -4756,7 +4768,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Oct 2023</t>
         </is>
@@ -4775,7 +4787,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Nov 2023</t>
         </is>
@@ -4794,7 +4806,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Dec 2023</t>
         </is>
@@ -4813,7 +4825,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Jan 2024</t>
         </is>
@@ -4832,7 +4844,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Feb 2024</t>
         </is>
@@ -4851,7 +4863,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Mar 2024</t>
         </is>
@@ -4870,7 +4882,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Apr 2024</t>
         </is>
@@ -4889,7 +4901,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>May 2024</t>
         </is>
@@ -4908,7 +4920,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Jun 2024</t>
         </is>
@@ -4927,7 +4939,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Jul 2024</t>
         </is>
@@ -4946,7 +4958,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Aug 2024</t>
         </is>
@@ -4965,7 +4977,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Sep 2024</t>
         </is>
@@ -4984,7 +4996,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Oct 2024</t>
         </is>
@@ -5003,7 +5015,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Nov 2024</t>
         </is>
@@ -5022,7 +5034,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
@@ -5041,7 +5053,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Jan 2025</t>
         </is>
@@ -5060,7 +5072,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>Feb 2025</t>
         </is>
@@ -5079,7 +5091,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>Mar 2025</t>
         </is>
@@ -5098,7 +5110,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Apr 2025</t>
         </is>
@@ -5117,7 +5129,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>May 2025</t>
         </is>
@@ -5136,7 +5148,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Jun 2025</t>
         </is>
@@ -5155,7 +5167,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="A35" s="17" t="inlineStr">
         <is>
           <t>Jul 2025</t>
         </is>
@@ -5174,7 +5186,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="inlineStr">
+      <c r="A36" s="17" t="inlineStr">
         <is>
           <t>Aug 2025</t>
         </is>
@@ -5193,7 +5205,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>Sep 2025</t>
         </is>
@@ -5212,7 +5224,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
@@ -5231,7 +5243,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>Nov 2025</t>
         </is>
@@ -5250,7 +5262,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>Dec 2025</t>
         </is>
@@ -5269,7 +5281,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>Jan 2026</t>
         </is>
@@ -5288,7 +5300,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="16" t="inlineStr">
+      <c r="A42" s="17" t="inlineStr">
         <is>
           <t>Feb 2026</t>
         </is>
@@ -5307,7 +5319,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
@@ -5326,7 +5338,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="16" t="inlineStr">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>Apr 2026</t>
         </is>
@@ -5345,7 +5357,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>May 2026</t>
         </is>
@@ -5364,7 +5376,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="16" t="inlineStr">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>Jun 2026</t>
         </is>

</xml_diff>

<commit_message>
Add 26 vs 24 change column to STR H1 comparison
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GzrfbzxdPZVRCw2bYpGG1J
</commit_message>
<xml_diff>
--- a/output/STR_Bangkok_by_segment_2023-2026.xlsx
+++ b/output/STR_Bangkok_by_segment_2023-2026.xlsx
@@ -1637,7 +1637,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>10</col>
+      <col>11</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -1659,7 +1659,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>10</col>
+      <col>11</col>
       <colOff>0</colOff>
       <row>19</row>
       <rowOff>0</rowOff>
@@ -1681,7 +1681,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>10</col>
+      <col>11</col>
       <colOff>0</colOff>
       <row>35</row>
       <rowOff>0</rowOff>
@@ -2074,7 +2074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2086,6 +2086,7 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2152,6 +2153,11 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
+          <t>26 vs 24</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
           <t>26 vs 23</t>
         </is>
       </c>
@@ -2184,6 +2190,9 @@
         <v>2.6</v>
       </c>
       <c r="I6" s="9" t="n">
+        <v>-8.199999999999999</v>
+      </c>
+      <c r="J6" s="9" t="n">
         <v>-0.7</v>
       </c>
     </row>
@@ -2215,6 +2224,9 @@
         <v>0.5</v>
       </c>
       <c r="I7" s="9" t="n">
+        <v>-10</v>
+      </c>
+      <c r="J7" s="9" t="n">
         <v>-2.9</v>
       </c>
     </row>
@@ -2245,7 +2257,10 @@
       <c r="H8" s="8" t="n">
         <v>5.1</v>
       </c>
-      <c r="I8" s="8" t="n">
+      <c r="I8" s="9" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="J8" s="8" t="n">
         <v>8.4</v>
       </c>
     </row>
@@ -2277,6 +2292,9 @@
         <v>3.4</v>
       </c>
       <c r="I9" s="8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J9" s="8" t="n">
         <v>9.300000000000001</v>
       </c>
     </row>
@@ -2330,6 +2348,11 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
+          <t>26 vs 24</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
           <t>26 vs 23</t>
         </is>
       </c>
@@ -2362,6 +2385,9 @@
         <v>1.1</v>
       </c>
       <c r="I22" s="8" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="J22" s="8" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2392,7 +2418,10 @@
       <c r="H23" s="9" t="n">
         <v>-2.9</v>
       </c>
-      <c r="I23" s="8" t="n">
+      <c r="I23" s="9" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="J23" s="8" t="n">
         <v>2.3</v>
       </c>
     </row>
@@ -2423,7 +2452,10 @@
       <c r="H24" s="9" t="n">
         <v>-4.5</v>
       </c>
-      <c r="I24" s="8" t="n">
+      <c r="I24" s="9" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="J24" s="8" t="n">
         <v>5.4</v>
       </c>
     </row>
@@ -2454,7 +2486,10 @@
       <c r="H25" s="9" t="n">
         <v>-7</v>
       </c>
-      <c r="I25" s="8" t="n">
+      <c r="I25" s="9" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="J25" s="8" t="n">
         <v>8.4</v>
       </c>
     </row>
@@ -2508,6 +2543,11 @@
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
+          <t>26 vs 24</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
           <t>26 vs 23</t>
         </is>
       </c>
@@ -2539,7 +2579,10 @@
       <c r="H38" s="8" t="n">
         <v>3.7</v>
       </c>
-      <c r="I38" s="8" t="n">
+      <c r="I38" s="9" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="J38" s="8" t="n">
         <v>6.2</v>
       </c>
     </row>
@@ -2571,6 +2614,9 @@
         <v>-2.4</v>
       </c>
       <c r="I39" s="9" t="n">
+        <v>-12</v>
+      </c>
+      <c r="J39" s="9" t="n">
         <v>-0.7</v>
       </c>
     </row>
@@ -2601,7 +2647,10 @@
       <c r="H40" s="8" t="n">
         <v>0.4</v>
       </c>
-      <c r="I40" s="8" t="n">
+      <c r="I40" s="9" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J40" s="8" t="n">
         <v>14.2</v>
       </c>
     </row>
@@ -2633,6 +2682,9 @@
         <v>-3.9</v>
       </c>
       <c r="I41" s="8" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J41" s="8" t="n">
         <v>18.4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Bangkok overall as full series to STR summary (monthly 2024-2026)
- New source: STR Bangkok market monthly 2024-2025.xls
- Bangkok overall in monthly sheets/charts (dashed gray, starts 2024),
  H1 tables with change columns where computable, YTD block, report

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GzrfbzxdPZVRCw2bYpGG1J
</commit_message>
<xml_diff>
--- a/output/STR_Bangkok_by_segment_2023-2026.xlsx
+++ b/output/STR_Bangkok_by_segment_2023-2026.xlsx
@@ -125,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -147,11 +147,14 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -406,6 +409,42 @@
             </strRef>
           </tx>
           <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="898781"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$5:$E$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$9:$E$9</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A10</f>
+            </strRef>
+          </tx>
+          <spPr>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -425,7 +464,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$9:$E$9</f>
+              <f>'Overview'!$B$10:$E$10</f>
             </numRef>
           </val>
         </ser>
@@ -640,6 +679,42 @@
             </strRef>
           </tx>
           <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="898781"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$21:$E$21</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$25:$E$25</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A26</f>
+            </strRef>
+          </tx>
+          <spPr>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -659,7 +734,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$25:$E$25</f>
+              <f>'Overview'!$B$26:$E$26</f>
             </numRef>
           </val>
         </ser>
@@ -874,6 +949,42 @@
             </strRef>
           </tx>
           <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="898781"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Overview'!$B$37:$E$37</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Overview'!$B$41:$E$41</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'Overview'!A42</f>
+            </strRef>
+          </tx>
+          <spPr>
             <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -893,7 +1004,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Overview'!$B$41:$E$41</f>
+              <f>'Overview'!$B$42:$E$42</f>
             </numRef>
           </val>
         </ser>
@@ -1096,6 +1207,42 @@
           <val>
             <numRef>
               <f>'Occupancy'!$E$5:$E$46</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Occupancy'!F4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="898781"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Occupancy'!$A$5:$A$46</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Occupancy'!$F$5:$F$46</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1333,6 +1480,42 @@
           </val>
           <smooth val="0"/>
         </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'ADR'!F4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="898781"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'ADR'!$A$5:$A$46</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'ADR'!$F$5:$F$46</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -1562,6 +1745,42 @@
           <val>
             <numRef>
               <f>'RevPAR'!$E$5:$E$46</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'RevPAR'!F4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="898781"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'RevPAR'!$A$5:$A$46</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'RevPAR'!$F$5:$F$46</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1708,7 +1927,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>7</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -1735,7 +1954,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>7</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -1762,7 +1981,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>7</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -2099,7 +2318,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>First-half (Jan–Jun) averages by market class, 2023–2026, with % change. Occupancy = %, ADR &amp; RevPAR = THB. ALL years calculated from STR monthly data (Occ/RevPAR day-weighted, ADR room-night-weighted) — STR's own YTD rows are not used (Mae's decision, 2026-08-03).</t>
+          <t>First-half (Jan–Jun) averages by market class, 2023–2026, with % change. Occupancy = %, ADR &amp; RevPAR = THB. ALL years calculated from STR monthly data (Occ/RevPAR day-weighted, ADR room-night-weighted) — STR's own YTD rows are not used (Mae's decision, 2026-08-03). Bangkok overall = whole market, data starts 2024.</t>
         </is>
       </c>
     </row>
@@ -2298,6 +2517,42 @@
         <v>9.300000000000001</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Bangkok overall</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n"/>
+      <c r="C10" s="7" t="n">
+        <v>73.7</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="J10" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -2363,16 +2618,16 @@
           <t>Luxury</t>
         </is>
       </c>
-      <c r="B22" s="13" t="n">
+      <c r="B22" s="16" t="n">
         <v>6620</v>
       </c>
-      <c r="C22" s="13" t="n">
+      <c r="C22" s="16" t="n">
         <v>6858</v>
       </c>
-      <c r="D22" s="13" t="n">
+      <c r="D22" s="16" t="n">
         <v>7007</v>
       </c>
-      <c r="E22" s="13" t="n">
+      <c r="E22" s="16" t="n">
         <v>7082</v>
       </c>
       <c r="F22" s="8" t="n">
@@ -2397,16 +2652,16 @@
           <t>Upper Upscale</t>
         </is>
       </c>
-      <c r="B23" s="13" t="n">
+      <c r="B23" s="16" t="n">
         <v>4205</v>
       </c>
-      <c r="C23" s="13" t="n">
+      <c r="C23" s="16" t="n">
         <v>4399</v>
       </c>
-      <c r="D23" s="13" t="n">
+      <c r="D23" s="16" t="n">
         <v>4430</v>
       </c>
-      <c r="E23" s="13" t="n">
+      <c r="E23" s="16" t="n">
         <v>4301</v>
       </c>
       <c r="F23" s="8" t="n">
@@ -2431,16 +2686,16 @@
           <t>Upscale</t>
         </is>
       </c>
-      <c r="B24" s="13" t="n">
+      <c r="B24" s="16" t="n">
         <v>2838</v>
       </c>
-      <c r="C24" s="13" t="n">
+      <c r="C24" s="16" t="n">
         <v>3038</v>
       </c>
-      <c r="D24" s="13" t="n">
+      <c r="D24" s="16" t="n">
         <v>3130</v>
       </c>
-      <c r="E24" s="13" t="n">
+      <c r="E24" s="16" t="n">
         <v>2991</v>
       </c>
       <c r="F24" s="8" t="n">
@@ -2465,16 +2720,16 @@
           <t>Upper Midscale</t>
         </is>
       </c>
-      <c r="B25" s="13" t="n">
+      <c r="B25" s="16" t="n">
         <v>2431</v>
       </c>
-      <c r="C25" s="13" t="n">
+      <c r="C25" s="16" t="n">
         <v>2697</v>
       </c>
-      <c r="D25" s="13" t="n">
+      <c r="D25" s="16" t="n">
         <v>2834</v>
       </c>
-      <c r="E25" s="13" t="n">
+      <c r="E25" s="16" t="n">
         <v>2635</v>
       </c>
       <c r="F25" s="8" t="n">
@@ -2493,6 +2748,42 @@
         <v>8.4</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>Bangkok overall</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="n"/>
+      <c r="C26" s="16" t="n">
+        <v>3960</v>
+      </c>
+      <c r="D26" s="16" t="n">
+        <v>4007</v>
+      </c>
+      <c r="E26" s="16" t="n">
+        <v>3952</v>
+      </c>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="I26" s="9" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="J26" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
@@ -2558,16 +2849,16 @@
           <t>Luxury</t>
         </is>
       </c>
-      <c r="B38" s="13" t="n">
+      <c r="B38" s="16" t="n">
         <v>4452</v>
       </c>
-      <c r="C38" s="13" t="n">
+      <c r="C38" s="16" t="n">
         <v>4987</v>
       </c>
-      <c r="D38" s="13" t="n">
+      <c r="D38" s="16" t="n">
         <v>4560</v>
       </c>
-      <c r="E38" s="13" t="n">
+      <c r="E38" s="16" t="n">
         <v>4729</v>
       </c>
       <c r="F38" s="8" t="n">
@@ -2592,16 +2883,16 @@
           <t>Upper Upscale</t>
         </is>
       </c>
-      <c r="B39" s="13" t="n">
+      <c r="B39" s="16" t="n">
         <v>2987</v>
       </c>
-      <c r="C39" s="13" t="n">
+      <c r="C39" s="16" t="n">
         <v>3369</v>
       </c>
-      <c r="D39" s="13" t="n">
+      <c r="D39" s="16" t="n">
         <v>3039</v>
       </c>
-      <c r="E39" s="13" t="n">
+      <c r="E39" s="16" t="n">
         <v>2965</v>
       </c>
       <c r="F39" s="8" t="n">
@@ -2626,16 +2917,16 @@
           <t>Upscale</t>
         </is>
       </c>
-      <c r="B40" s="13" t="n">
+      <c r="B40" s="16" t="n">
         <v>1975</v>
       </c>
-      <c r="C40" s="13" t="n">
+      <c r="C40" s="16" t="n">
         <v>2301</v>
       </c>
-      <c r="D40" s="13" t="n">
+      <c r="D40" s="16" t="n">
         <v>2247</v>
       </c>
-      <c r="E40" s="13" t="n">
+      <c r="E40" s="16" t="n">
         <v>2256</v>
       </c>
       <c r="F40" s="8" t="n">
@@ -2660,16 +2951,16 @@
           <t>Upper Midscale</t>
         </is>
       </c>
-      <c r="B41" s="13" t="n">
+      <c r="B41" s="16" t="n">
         <v>1710</v>
       </c>
-      <c r="C41" s="13" t="n">
+      <c r="C41" s="16" t="n">
         <v>2003</v>
       </c>
-      <c r="D41" s="13" t="n">
+      <c r="D41" s="16" t="n">
         <v>2106</v>
       </c>
-      <c r="E41" s="13" t="n">
+      <c r="E41" s="16" t="n">
         <v>2024</v>
       </c>
       <c r="F41" s="8" t="n">
@@ -2688,6 +2979,42 @@
         <v>18.4</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>Bangkok overall</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="n"/>
+      <c r="C42" s="16" t="n">
+        <v>2921</v>
+      </c>
+      <c r="D42" s="16" t="n">
+        <v>2762</v>
+      </c>
+      <c r="E42" s="16" t="n">
+        <v>2787</v>
+      </c>
+      <c r="F42" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="H42" s="8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I42" s="9" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="J42" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
@@ -2733,7 +3060,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="14" t="inlineStr">
+      <c r="A54" s="13" t="inlineStr">
         <is>
           <t>Bangkok overall</t>
         </is>
@@ -2741,26 +3068,20 @@
       <c r="B54" s="7" t="n">
         <v>70.5</v>
       </c>
-      <c r="C54" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D54" s="13" t="n">
+      <c r="C54" s="8" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="D54" s="16" t="n">
         <v>3952</v>
       </c>
-      <c r="E54" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F54" s="13" t="n">
+      <c r="E54" s="9" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="F54" s="16" t="n">
         <v>2787</v>
       </c>
-      <c r="G54" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="G54" s="8" t="n">
+        <v>0.9</v>
       </c>
     </row>
     <row r="55">
@@ -2775,13 +3096,13 @@
       <c r="C55" s="8" t="n">
         <v>2.6</v>
       </c>
-      <c r="D55" s="13" t="n">
+      <c r="D55" s="16" t="n">
         <v>7082</v>
       </c>
       <c r="E55" s="8" t="n">
         <v>1.1</v>
       </c>
-      <c r="F55" s="13" t="n">
+      <c r="F55" s="16" t="n">
         <v>4729</v>
       </c>
       <c r="G55" s="8" t="n">
@@ -2800,13 +3121,13 @@
       <c r="C56" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="D56" s="13" t="n">
+      <c r="D56" s="16" t="n">
         <v>4301</v>
       </c>
       <c r="E56" s="9" t="n">
         <v>-2.9</v>
       </c>
-      <c r="F56" s="13" t="n">
+      <c r="F56" s="16" t="n">
         <v>2965</v>
       </c>
       <c r="G56" s="9" t="n">
@@ -2825,13 +3146,13 @@
       <c r="C57" s="8" t="n">
         <v>5.1</v>
       </c>
-      <c r="D57" s="13" t="n">
+      <c r="D57" s="16" t="n">
         <v>2991</v>
       </c>
       <c r="E57" s="9" t="n">
         <v>-4.5</v>
       </c>
-      <c r="F57" s="13" t="n">
+      <c r="F57" s="16" t="n">
         <v>2256</v>
       </c>
       <c r="G57" s="8" t="n">
@@ -2850,13 +3171,13 @@
       <c r="C58" s="8" t="n">
         <v>3.4</v>
       </c>
-      <c r="D58" s="13" t="n">
+      <c r="D58" s="16" t="n">
         <v>2635</v>
       </c>
       <c r="E58" s="9" t="n">
         <v>-7</v>
       </c>
-      <c r="F58" s="13" t="n">
+      <c r="F58" s="16" t="n">
         <v>2024</v>
       </c>
       <c r="G58" s="9" t="n">
@@ -2875,7 +3196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2883,10 +3204,11 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Bangkok STR — Occupancy by market class (monthly, This Year)</t>
         </is>
@@ -2925,9 +3247,14 @@
           <t>Upper Midscale</t>
         </is>
       </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Bangkok overall</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>Jan 2023</t>
         </is>
@@ -2944,9 +3271,10 @@
       <c r="E5" s="7" t="n">
         <v>69.81</v>
       </c>
+      <c r="F5" s="14" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Feb 2023</t>
         </is>
@@ -2963,9 +3291,10 @@
       <c r="E6" s="7" t="n">
         <v>74.95</v>
       </c>
+      <c r="F6" s="14" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Mar 2023</t>
         </is>
@@ -2982,9 +3311,10 @@
       <c r="E7" s="7" t="n">
         <v>74.15000000000001</v>
       </c>
+      <c r="F7" s="14" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Apr 2023</t>
         </is>
@@ -3001,9 +3331,10 @@
       <c r="E8" s="7" t="n">
         <v>68.75</v>
       </c>
+      <c r="F8" s="14" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>May 2023</t>
         </is>
@@ -3020,9 +3351,10 @@
       <c r="E9" s="7" t="n">
         <v>66.67</v>
       </c>
+      <c r="F9" s="14" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Jun 2023</t>
         </is>
@@ -3039,9 +3371,10 @@
       <c r="E10" s="7" t="n">
         <v>67.95</v>
       </c>
+      <c r="F10" s="14" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>Jul 2023</t>
         </is>
@@ -3058,9 +3391,10 @@
       <c r="E11" s="7" t="n">
         <v>73</v>
       </c>
+      <c r="F11" s="14" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Aug 2023</t>
         </is>
@@ -3077,9 +3411,10 @@
       <c r="E12" s="7" t="n">
         <v>75</v>
       </c>
+      <c r="F12" s="14" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Sep 2023</t>
         </is>
@@ -3096,9 +3431,10 @@
       <c r="E13" s="7" t="n">
         <v>70.61</v>
       </c>
+      <c r="F13" s="14" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Oct 2023</t>
         </is>
@@ -3115,9 +3451,10 @@
       <c r="E14" s="7" t="n">
         <v>67.67</v>
       </c>
+      <c r="F14" s="14" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>Nov 2023</t>
         </is>
@@ -3134,9 +3471,10 @@
       <c r="E15" s="7" t="n">
         <v>76.36</v>
       </c>
+      <c r="F15" s="14" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Dec 2023</t>
         </is>
@@ -3153,9 +3491,10 @@
       <c r="E16" s="7" t="n">
         <v>76.03</v>
       </c>
+      <c r="F16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>Jan 2024</t>
         </is>
@@ -3172,9 +3511,12 @@
       <c r="E17" s="7" t="n">
         <v>76.55</v>
       </c>
+      <c r="F17" s="7" t="n">
+        <v>73.42</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Feb 2024</t>
         </is>
@@ -3191,9 +3533,12 @@
       <c r="E18" s="7" t="n">
         <v>79.95</v>
       </c>
+      <c r="F18" s="7" t="n">
+        <v>81.3</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Mar 2024</t>
         </is>
@@ -3210,9 +3555,12 @@
       <c r="E19" s="7" t="n">
         <v>73.69</v>
       </c>
+      <c r="F19" s="7" t="n">
+        <v>73.53</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>Apr 2024</t>
         </is>
@@ -3229,9 +3577,12 @@
       <c r="E20" s="7" t="n">
         <v>70.56</v>
       </c>
+      <c r="F20" s="7" t="n">
+        <v>70.7</v>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>May 2024</t>
         </is>
@@ -3248,9 +3599,12 @@
       <c r="E21" s="7" t="n">
         <v>71.31999999999999</v>
       </c>
+      <c r="F21" s="7" t="n">
+        <v>70.52</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>Jun 2024</t>
         </is>
@@ -3267,9 +3621,12 @@
       <c r="E22" s="7" t="n">
         <v>73.77</v>
       </c>
+      <c r="F22" s="7" t="n">
+        <v>73.40000000000001</v>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>Jul 2024</t>
         </is>
@@ -3286,9 +3643,12 @@
       <c r="E23" s="7" t="n">
         <v>79.7</v>
       </c>
+      <c r="F23" s="7" t="n">
+        <v>77.79000000000001</v>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>Aug 2024</t>
         </is>
@@ -3305,9 +3665,12 @@
       <c r="E24" s="7" t="n">
         <v>81.28</v>
       </c>
+      <c r="F24" s="7" t="n">
+        <v>79.28</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>Sep 2024</t>
         </is>
@@ -3324,9 +3687,12 @@
       <c r="E25" s="7" t="n">
         <v>71.95</v>
       </c>
+      <c r="F25" s="7" t="n">
+        <v>67.19</v>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>Oct 2024</t>
         </is>
@@ -3343,9 +3709,12 @@
       <c r="E26" s="7" t="n">
         <v>71.48999999999999</v>
       </c>
+      <c r="F26" s="7" t="n">
+        <v>67.15000000000001</v>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="inlineStr">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>Nov 2024</t>
         </is>
@@ -3362,9 +3731,12 @@
       <c r="E27" s="7" t="n">
         <v>84.05</v>
       </c>
+      <c r="F27" s="7" t="n">
+        <v>81.97</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="inlineStr">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
@@ -3381,9 +3753,12 @@
       <c r="E28" s="7" t="n">
         <v>82.09999999999999</v>
       </c>
+      <c r="F28" s="7" t="n">
+        <v>78.89</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="inlineStr">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>Jan 2025</t>
         </is>
@@ -3400,9 +3775,12 @@
       <c r="E29" s="7" t="n">
         <v>80.94</v>
       </c>
+      <c r="F29" s="7" t="n">
+        <v>77.52</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="inlineStr">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>Feb 2025</t>
         </is>
@@ -3419,9 +3797,12 @@
       <c r="E30" s="7" t="n">
         <v>82.70999999999999</v>
       </c>
+      <c r="F30" s="7" t="n">
+        <v>78.64</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="inlineStr">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>Mar 2025</t>
         </is>
@@ -3438,9 +3819,12 @@
       <c r="E31" s="7" t="n">
         <v>74.20999999999999</v>
       </c>
+      <c r="F31" s="7" t="n">
+        <v>68.81999999999999</v>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="17" t="inlineStr">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>Apr 2025</t>
         </is>
@@ -3457,9 +3841,12 @@
       <c r="E32" s="7" t="n">
         <v>67.98999999999999</v>
       </c>
+      <c r="F32" s="7" t="n">
+        <v>62.29</v>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>May 2025</t>
         </is>
@@ -3476,9 +3863,12 @@
       <c r="E33" s="7" t="n">
         <v>70.37</v>
       </c>
+      <c r="F33" s="7" t="n">
+        <v>63.27</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="inlineStr">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>Jun 2025</t>
         </is>
@@ -3495,9 +3885,12 @@
       <c r="E34" s="7" t="n">
         <v>70.09</v>
       </c>
+      <c r="F34" s="7" t="n">
+        <v>63.65</v>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="inlineStr">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>Jul 2025</t>
         </is>
@@ -3514,9 +3907,12 @@
       <c r="E35" s="7" t="n">
         <v>76.69</v>
       </c>
+      <c r="F35" s="7" t="n">
+        <v>69.70999999999999</v>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="17" t="inlineStr">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>Aug 2025</t>
         </is>
@@ -3533,9 +3929,12 @@
       <c r="E36" s="7" t="n">
         <v>79.09</v>
       </c>
+      <c r="F36" s="7" t="n">
+        <v>72.75</v>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="inlineStr">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>Sep 2025</t>
         </is>
@@ -3552,9 +3951,12 @@
       <c r="E37" s="7" t="n">
         <v>70.31999999999999</v>
       </c>
+      <c r="F37" s="7" t="n">
+        <v>64.11</v>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="inlineStr">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
@@ -3571,9 +3973,12 @@
       <c r="E38" s="7" t="n">
         <v>74.28</v>
       </c>
+      <c r="F38" s="7" t="n">
+        <v>68.73999999999999</v>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="17" t="inlineStr">
+      <c r="A39" s="18" t="inlineStr">
         <is>
           <t>Nov 2025</t>
         </is>
@@ -3590,9 +3995,12 @@
       <c r="E39" s="7" t="n">
         <v>84.03</v>
       </c>
+      <c r="F39" s="7" t="n">
+        <v>79.06</v>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="inlineStr">
+      <c r="A40" s="18" t="inlineStr">
         <is>
           <t>Dec 2025</t>
         </is>
@@ -3609,9 +4017,12 @@
       <c r="E40" s="7" t="n">
         <v>80.59999999999999</v>
       </c>
+      <c r="F40" s="7" t="n">
+        <v>76.90000000000001</v>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="17" t="inlineStr">
+      <c r="A41" s="18" t="inlineStr">
         <is>
           <t>Jan 2026</t>
         </is>
@@ -3628,9 +4039,12 @@
       <c r="E41" s="7" t="n">
         <v>80.59</v>
       </c>
+      <c r="F41" s="7" t="n">
+        <v>75.69</v>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="17" t="inlineStr">
+      <c r="A42" s="18" t="inlineStr">
         <is>
           <t>Feb 2026</t>
         </is>
@@ -3647,9 +4061,12 @@
       <c r="E42" s="7" t="n">
         <v>86.25</v>
       </c>
+      <c r="F42" s="7" t="n">
+        <v>80.86</v>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="inlineStr">
+      <c r="A43" s="18" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
@@ -3666,9 +4083,12 @@
       <c r="E43" s="7" t="n">
         <v>79.8</v>
       </c>
+      <c r="F43" s="7" t="n">
+        <v>73.25</v>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+      <c r="A44" s="18" t="inlineStr">
         <is>
           <t>Apr 2026</t>
         </is>
@@ -3685,9 +4105,12 @@
       <c r="E44" s="7" t="n">
         <v>70.38</v>
       </c>
+      <c r="F44" s="7" t="n">
+        <v>64.67</v>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="17" t="inlineStr">
+      <c r="A45" s="18" t="inlineStr">
         <is>
           <t>May 2026</t>
         </is>
@@ -3704,9 +4127,12 @@
       <c r="E45" s="7" t="n">
         <v>71.84</v>
       </c>
+      <c r="F45" s="7" t="n">
+        <v>65.36</v>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="17" t="inlineStr">
+      <c r="A46" s="18" t="inlineStr">
         <is>
           <t>Jun 2026</t>
         </is>
@@ -3722,6 +4148,9 @@
       </c>
       <c r="E46" s="7" t="n">
         <v>72.70999999999999</v>
+      </c>
+      <c r="F46" s="7" t="n">
+        <v>63.87</v>
       </c>
     </row>
   </sheetData>
@@ -3736,7 +4165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3744,10 +4173,11 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Bangkok STR — ADR by market class (monthly, This Year)</t>
         </is>
@@ -3786,803 +4216,910 @@
           <t>Upper Midscale</t>
         </is>
       </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Bangkok overall</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>Jan 2023</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="16" t="n">
         <v>7257.67</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="16" t="n">
         <v>4324.77</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="16" t="n">
         <v>2863.43</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="16" t="n">
         <v>2469.09</v>
       </c>
+      <c r="F5" s="14" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Feb 2023</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="16" t="n">
         <v>6650.01</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="16" t="n">
         <v>4201.15</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="16" t="n">
         <v>2829.5</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="16" t="n">
         <v>2395.04</v>
       </c>
+      <c r="F6" s="14" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Mar 2023</t>
         </is>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="16" t="n">
         <v>6489.71</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="16" t="n">
         <v>4235.39</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="16" t="n">
         <v>2890.68</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="16" t="n">
         <v>2443.81</v>
       </c>
+      <c r="F7" s="14" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Apr 2023</t>
         </is>
       </c>
-      <c r="B8" s="13" t="n">
+      <c r="B8" s="16" t="n">
         <v>6949.89</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="16" t="n">
         <v>4309.86</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="16" t="n">
         <v>2879.78</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="16" t="n">
         <v>2485.27</v>
       </c>
+      <c r="F8" s="14" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>May 2023</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="16" t="n">
         <v>6174.16</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="16" t="n">
         <v>4063.43</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="16" t="n">
         <v>2745.19</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="16" t="n">
         <v>2357.71</v>
       </c>
+      <c r="F9" s="14" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Jun 2023</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n">
+      <c r="B10" s="16" t="n">
         <v>6145.31</v>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="16" t="n">
         <v>4084.32</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="16" t="n">
         <v>2815.39</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="16" t="n">
         <v>2434.92</v>
       </c>
+      <c r="F10" s="14" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>Jul 2023</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" s="16" t="n">
         <v>6593.69</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="16" t="n">
         <v>4220.41</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="16" t="n">
         <v>2974.75</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="16" t="n">
         <v>2560.81</v>
       </c>
+      <c r="F11" s="14" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Aug 2023</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n">
+      <c r="B12" s="16" t="n">
         <v>6499</v>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="16" t="n">
         <v>4222.3</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="16" t="n">
         <v>2937.66</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="16" t="n">
         <v>2612.55</v>
       </c>
+      <c r="F12" s="14" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Sep 2023</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="B13" s="16" t="n">
         <v>6004.24</v>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="16" t="n">
         <v>4003.59</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="16" t="n">
         <v>2747.58</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="16" t="n">
         <v>2515.08</v>
       </c>
+      <c r="F13" s="14" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Oct 2023</t>
         </is>
       </c>
-      <c r="B14" s="13" t="n">
+      <c r="B14" s="16" t="n">
         <v>6310.62</v>
       </c>
-      <c r="C14" s="13" t="n">
+      <c r="C14" s="16" t="n">
         <v>4070.44</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="16" t="n">
         <v>2760.38</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="16" t="n">
         <v>2482.23</v>
       </c>
+      <c r="F14" s="14" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>Nov 2023</t>
         </is>
       </c>
-      <c r="B15" s="13" t="n">
+      <c r="B15" s="16" t="n">
         <v>6636.91</v>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C15" s="16" t="n">
         <v>4332.99</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="16" t="n">
         <v>2984.16</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="16" t="n">
         <v>2682.9</v>
       </c>
+      <c r="F15" s="14" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Dec 2023</t>
         </is>
       </c>
-      <c r="B16" s="13" t="n">
+      <c r="B16" s="16" t="n">
         <v>8183.87</v>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C16" s="16" t="n">
         <v>4906.12</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="16" t="n">
         <v>3341.61</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="16" t="n">
         <v>3038.37</v>
       </c>
+      <c r="F16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>Jan 2024</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n">
+      <c r="B17" s="16" t="n">
         <v>7232.85</v>
       </c>
-      <c r="C17" s="13" t="n">
+      <c r="C17" s="16" t="n">
         <v>4449.88</v>
       </c>
-      <c r="D17" s="13" t="n">
+      <c r="D17" s="16" t="n">
         <v>3027</v>
       </c>
-      <c r="E17" s="13" t="n">
+      <c r="E17" s="16" t="n">
         <v>2695.29</v>
       </c>
+      <c r="F17" s="16" t="n">
+        <v>4080.14</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Feb 2024</t>
         </is>
       </c>
-      <c r="B18" s="13" t="n">
+      <c r="B18" s="16" t="n">
         <v>7511.89</v>
       </c>
-      <c r="C18" s="13" t="n">
+      <c r="C18" s="16" t="n">
         <v>4711.27</v>
       </c>
-      <c r="D18" s="13" t="n">
+      <c r="D18" s="16" t="n">
         <v>3259.63</v>
       </c>
-      <c r="E18" s="13" t="n">
+      <c r="E18" s="16" t="n">
         <v>2876.63</v>
       </c>
+      <c r="F18" s="16" t="n">
+        <v>4315.26</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Mar 2024</t>
         </is>
       </c>
-      <c r="B19" s="13" t="n">
+      <c r="B19" s="16" t="n">
         <v>6678.36</v>
       </c>
-      <c r="C19" s="13" t="n">
+      <c r="C19" s="16" t="n">
         <v>4349.05</v>
       </c>
-      <c r="D19" s="13" t="n">
+      <c r="D19" s="16" t="n">
         <v>3000.15</v>
       </c>
-      <c r="E19" s="13" t="n">
+      <c r="E19" s="16" t="n">
         <v>2661.83</v>
       </c>
+      <c r="F19" s="16" t="n">
+        <v>3879.63</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>Apr 2024</t>
         </is>
       </c>
-      <c r="B20" s="13" t="n">
+      <c r="B20" s="16" t="n">
         <v>6807.84</v>
       </c>
-      <c r="C20" s="13" t="n">
+      <c r="C20" s="16" t="n">
         <v>4374.91</v>
       </c>
-      <c r="D20" s="13" t="n">
+      <c r="D20" s="16" t="n">
         <v>3020.58</v>
       </c>
-      <c r="E20" s="13" t="n">
+      <c r="E20" s="16" t="n">
         <v>2684.7</v>
       </c>
+      <c r="F20" s="16" t="n">
+        <v>3923.77</v>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>May 2024</t>
         </is>
       </c>
-      <c r="B21" s="13" t="n">
+      <c r="B21" s="16" t="n">
         <v>6383.14</v>
       </c>
-      <c r="C21" s="13" t="n">
+      <c r="C21" s="16" t="n">
         <v>4216.76</v>
       </c>
-      <c r="D21" s="13" t="n">
+      <c r="D21" s="16" t="n">
         <v>2910.82</v>
       </c>
-      <c r="E21" s="13" t="n">
+      <c r="E21" s="16" t="n">
         <v>2589.48</v>
       </c>
+      <c r="F21" s="16" t="n">
+        <v>3720.21</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>Jun 2024</t>
         </is>
       </c>
-      <c r="B22" s="13" t="n">
+      <c r="B22" s="16" t="n">
         <v>6435.11</v>
       </c>
-      <c r="C22" s="13" t="n">
+      <c r="C22" s="16" t="n">
         <v>4256.48</v>
       </c>
-      <c r="D22" s="13" t="n">
+      <c r="D22" s="16" t="n">
         <v>2996.93</v>
       </c>
-      <c r="E22" s="13" t="n">
+      <c r="E22" s="16" t="n">
         <v>2667.56</v>
       </c>
+      <c r="F22" s="16" t="n">
+        <v>3813.5</v>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>Jul 2024</t>
         </is>
       </c>
-      <c r="B23" s="13" t="n">
+      <c r="B23" s="16" t="n">
         <v>6765.18</v>
       </c>
-      <c r="C23" s="13" t="n">
+      <c r="C23" s="16" t="n">
         <v>4405.22</v>
       </c>
-      <c r="D23" s="13" t="n">
+      <c r="D23" s="16" t="n">
         <v>3138.3</v>
       </c>
-      <c r="E23" s="13" t="n">
+      <c r="E23" s="16" t="n">
         <v>2803.39</v>
       </c>
+      <c r="F23" s="16" t="n">
+        <v>3988.07</v>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>Aug 2024</t>
         </is>
       </c>
-      <c r="B24" s="13" t="n">
+      <c r="B24" s="16" t="n">
         <v>6914.04</v>
       </c>
-      <c r="C24" s="13" t="n">
+      <c r="C24" s="16" t="n">
         <v>4556.91</v>
       </c>
-      <c r="D24" s="13" t="n">
+      <c r="D24" s="16" t="n">
         <v>3238.95</v>
       </c>
-      <c r="E24" s="13" t="n">
+      <c r="E24" s="16" t="n">
         <v>2908.9</v>
       </c>
+      <c r="F24" s="16" t="n">
+        <v>4111.42</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>Sep 2024</t>
         </is>
       </c>
-      <c r="B25" s="13" t="n">
+      <c r="B25" s="16" t="n">
         <v>6115.68</v>
       </c>
-      <c r="C25" s="13" t="n">
+      <c r="C25" s="16" t="n">
         <v>4132.36</v>
       </c>
-      <c r="D25" s="13" t="n">
+      <c r="D25" s="16" t="n">
         <v>2912.96</v>
       </c>
-      <c r="E25" s="13" t="n">
+      <c r="E25" s="16" t="n">
         <v>2673.8</v>
       </c>
+      <c r="F25" s="16" t="n">
+        <v>3660.29</v>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>Oct 2024</t>
         </is>
       </c>
-      <c r="B26" s="13" t="n">
+      <c r="B26" s="16" t="n">
         <v>6438.59</v>
       </c>
-      <c r="C26" s="13" t="n">
+      <c r="C26" s="16" t="n">
         <v>4174.16</v>
       </c>
-      <c r="D26" s="13" t="n">
+      <c r="D26" s="16" t="n">
         <v>2938.5</v>
       </c>
-      <c r="E26" s="13" t="n">
+      <c r="E26" s="16" t="n">
         <v>2709.8</v>
       </c>
+      <c r="F26" s="16" t="n">
+        <v>3776.9</v>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="inlineStr">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>Nov 2024</t>
         </is>
       </c>
-      <c r="B27" s="13" t="n">
+      <c r="B27" s="16" t="n">
         <v>7230.78</v>
       </c>
-      <c r="C27" s="13" t="n">
+      <c r="C27" s="16" t="n">
         <v>4771.42</v>
       </c>
-      <c r="D27" s="13" t="n">
+      <c r="D27" s="16" t="n">
         <v>3413.37</v>
       </c>
-      <c r="E27" s="13" t="n">
+      <c r="E27" s="16" t="n">
         <v>3097.43</v>
       </c>
+      <c r="F27" s="16" t="n">
+        <v>4344.69</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="inlineStr">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
       </c>
-      <c r="B28" s="13" t="n">
+      <c r="B28" s="16" t="n">
         <v>8865.09</v>
       </c>
-      <c r="C28" s="13" t="n">
+      <c r="C28" s="16" t="n">
         <v>5305.73</v>
       </c>
-      <c r="D28" s="13" t="n">
+      <c r="D28" s="16" t="n">
         <v>3776.59</v>
       </c>
-      <c r="E28" s="13" t="n">
+      <c r="E28" s="16" t="n">
         <v>3466.66</v>
       </c>
+      <c r="F28" s="16" t="n">
+        <v>5004.38</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="inlineStr">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>Jan 2025</t>
         </is>
       </c>
-      <c r="B29" s="13" t="n">
+      <c r="B29" s="16" t="n">
         <v>8155.43</v>
       </c>
-      <c r="C29" s="13" t="n">
+      <c r="C29" s="16" t="n">
         <v>4881.25</v>
       </c>
-      <c r="D29" s="13" t="n">
+      <c r="D29" s="16" t="n">
         <v>3479.24</v>
       </c>
-      <c r="E29" s="13" t="n">
+      <c r="E29" s="16" t="n">
         <v>3216.07</v>
       </c>
+      <c r="F29" s="16" t="n">
+        <v>4605.45</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="inlineStr">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>Feb 2025</t>
         </is>
       </c>
-      <c r="B30" s="13" t="n">
+      <c r="B30" s="16" t="n">
         <v>7324.96</v>
       </c>
-      <c r="C30" s="13" t="n">
+      <c r="C30" s="16" t="n">
         <v>4680.93</v>
       </c>
-      <c r="D30" s="13" t="n">
+      <c r="D30" s="16" t="n">
         <v>3329.91</v>
       </c>
-      <c r="E30" s="13" t="n">
+      <c r="E30" s="16" t="n">
         <v>3048.34</v>
       </c>
+      <c r="F30" s="16" t="n">
+        <v>4286.41</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="inlineStr">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>Mar 2025</t>
         </is>
       </c>
-      <c r="B31" s="13" t="n">
+      <c r="B31" s="16" t="n">
         <v>6728.43</v>
       </c>
-      <c r="C31" s="13" t="n">
+      <c r="C31" s="16" t="n">
         <v>4343.3</v>
       </c>
-      <c r="D31" s="13" t="n">
+      <c r="D31" s="16" t="n">
         <v>3091.87</v>
       </c>
-      <c r="E31" s="13" t="n">
+      <c r="E31" s="16" t="n">
         <v>2805.96</v>
       </c>
+      <c r="F31" s="16" t="n">
+        <v>3890.63</v>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="17" t="inlineStr">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>Apr 2025</t>
         </is>
       </c>
-      <c r="B32" s="13" t="n">
+      <c r="B32" s="16" t="n">
         <v>6827.43</v>
       </c>
-      <c r="C32" s="13" t="n">
+      <c r="C32" s="16" t="n">
         <v>4265.86</v>
       </c>
-      <c r="D32" s="13" t="n">
+      <c r="D32" s="16" t="n">
         <v>3038.34</v>
       </c>
-      <c r="E32" s="13" t="n">
+      <c r="E32" s="16" t="n">
         <v>2694.61</v>
       </c>
+      <c r="F32" s="16" t="n">
+        <v>3869</v>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>May 2025</t>
         </is>
       </c>
-      <c r="B33" s="13" t="n">
+      <c r="B33" s="16" t="n">
         <v>6332.58</v>
       </c>
-      <c r="C33" s="13" t="n">
+      <c r="C33" s="16" t="n">
         <v>4184.04</v>
       </c>
-      <c r="D33" s="13" t="n">
+      <c r="D33" s="16" t="n">
         <v>2877.48</v>
       </c>
-      <c r="E33" s="13" t="n">
+      <c r="E33" s="16" t="n">
         <v>2573.31</v>
       </c>
+      <c r="F33" s="16" t="n">
+        <v>3638.97</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="inlineStr">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>Jun 2025</t>
         </is>
       </c>
-      <c r="B34" s="13" t="n">
+      <c r="B34" s="16" t="n">
         <v>6218.14</v>
       </c>
-      <c r="C34" s="13" t="n">
+      <c r="C34" s="16" t="n">
         <v>4068.12</v>
       </c>
-      <c r="D34" s="13" t="n">
+      <c r="D34" s="16" t="n">
         <v>2885.56</v>
       </c>
-      <c r="E34" s="13" t="n">
+      <c r="E34" s="16" t="n">
         <v>2576.24</v>
       </c>
+      <c r="F34" s="16" t="n">
+        <v>3572.01</v>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="inlineStr">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>Jul 2025</t>
         </is>
       </c>
-      <c r="B35" s="13" t="n">
+      <c r="B35" s="16" t="n">
         <v>6563.5</v>
       </c>
-      <c r="C35" s="13" t="n">
+      <c r="C35" s="16" t="n">
         <v>4170.97</v>
       </c>
-      <c r="D35" s="13" t="n">
+      <c r="D35" s="16" t="n">
         <v>3010.69</v>
       </c>
-      <c r="E35" s="13" t="n">
+      <c r="E35" s="16" t="n">
         <v>2707.91</v>
       </c>
+      <c r="F35" s="16" t="n">
+        <v>3769.59</v>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="17" t="inlineStr">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>Aug 2025</t>
         </is>
       </c>
-      <c r="B36" s="13" t="n">
+      <c r="B36" s="16" t="n">
         <v>6631.46</v>
       </c>
-      <c r="C36" s="13" t="n">
+      <c r="C36" s="16" t="n">
         <v>4168.19</v>
       </c>
-      <c r="D36" s="13" t="n">
+      <c r="D36" s="16" t="n">
         <v>3034.68</v>
       </c>
-      <c r="E36" s="13" t="n">
+      <c r="E36" s="16" t="n">
         <v>2758.53</v>
       </c>
+      <c r="F36" s="16" t="n">
+        <v>3819.7</v>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="inlineStr">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>Sep 2025</t>
         </is>
       </c>
-      <c r="B37" s="13" t="n">
+      <c r="B37" s="16" t="n">
         <v>5950.24</v>
       </c>
-      <c r="C37" s="13" t="n">
+      <c r="C37" s="16" t="n">
         <v>3898.96</v>
       </c>
-      <c r="D37" s="13" t="n">
+      <c r="D37" s="16" t="n">
         <v>2773.08</v>
       </c>
-      <c r="E37" s="13" t="n">
+      <c r="E37" s="16" t="n">
         <v>2519.21</v>
       </c>
+      <c r="F37" s="16" t="n">
+        <v>3430.29</v>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="inlineStr">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
       </c>
-      <c r="B38" s="13" t="n">
+      <c r="B38" s="16" t="n">
         <v>6476.21</v>
       </c>
-      <c r="C38" s="13" t="n">
+      <c r="C38" s="16" t="n">
         <v>4096.54</v>
       </c>
-      <c r="D38" s="13" t="n">
+      <c r="D38" s="16" t="n">
         <v>2833.55</v>
       </c>
-      <c r="E38" s="13" t="n">
+      <c r="E38" s="16" t="n">
         <v>2628.42</v>
       </c>
+      <c r="F38" s="16" t="n">
+        <v>3707.04</v>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="17" t="inlineStr">
+      <c r="A39" s="18" t="inlineStr">
         <is>
           <t>Nov 2025</t>
         </is>
       </c>
-      <c r="B39" s="13" t="n">
+      <c r="B39" s="16" t="n">
         <v>6973.41</v>
       </c>
-      <c r="C39" s="13" t="n">
+      <c r="C39" s="16" t="n">
         <v>4483.61</v>
       </c>
-      <c r="D39" s="13" t="n">
+      <c r="D39" s="16" t="n">
         <v>3125.73</v>
       </c>
-      <c r="E39" s="13" t="n">
+      <c r="E39" s="16" t="n">
         <v>2849.07</v>
       </c>
+      <c r="F39" s="16" t="n">
+        <v>4043.87</v>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="inlineStr">
+      <c r="A40" s="18" t="inlineStr">
         <is>
           <t>Dec 2025</t>
         </is>
       </c>
-      <c r="B40" s="13" t="n">
+      <c r="B40" s="16" t="n">
         <v>8911.91</v>
       </c>
-      <c r="C40" s="13" t="n">
+      <c r="C40" s="16" t="n">
         <v>5153.75</v>
       </c>
-      <c r="D40" s="13" t="n">
+      <c r="D40" s="16" t="n">
         <v>3562.61</v>
       </c>
-      <c r="E40" s="13" t="n">
+      <c r="E40" s="16" t="n">
         <v>3246.97</v>
       </c>
+      <c r="F40" s="16" t="n">
+        <v>4862.19</v>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="17" t="inlineStr">
+      <c r="A41" s="18" t="inlineStr">
         <is>
           <t>Jan 2026</t>
         </is>
       </c>
-      <c r="B41" s="13" t="n">
+      <c r="B41" s="16" t="n">
         <v>7720.67</v>
       </c>
-      <c r="C41" s="13" t="n">
+      <c r="C41" s="16" t="n">
         <v>4576.36</v>
       </c>
-      <c r="D41" s="13" t="n">
+      <c r="D41" s="16" t="n">
         <v>3212.95</v>
       </c>
-      <c r="E41" s="13" t="n">
+      <c r="E41" s="16" t="n">
         <v>2895.57</v>
       </c>
+      <c r="F41" s="16" t="n">
+        <v>4279.7</v>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="17" t="inlineStr">
+      <c r="A42" s="18" t="inlineStr">
         <is>
           <t>Feb 2026</t>
         </is>
       </c>
-      <c r="B42" s="13" t="n">
+      <c r="B42" s="16" t="n">
         <v>7628.74</v>
       </c>
-      <c r="C42" s="13" t="n">
+      <c r="C42" s="16" t="n">
         <v>4627.26</v>
       </c>
-      <c r="D42" s="13" t="n">
+      <c r="D42" s="16" t="n">
         <v>3271.69</v>
       </c>
-      <c r="E42" s="13" t="n">
+      <c r="E42" s="16" t="n">
         <v>2899.86</v>
       </c>
+      <c r="F42" s="16" t="n">
+        <v>4348.93</v>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="inlineStr">
+      <c r="A43" s="18" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="B43" s="13" t="n">
+      <c r="B43" s="16" t="n">
         <v>7037.04</v>
       </c>
-      <c r="C43" s="13" t="n">
+      <c r="C43" s="16" t="n">
         <v>4298.88</v>
       </c>
-      <c r="D43" s="13" t="n">
+      <c r="D43" s="16" t="n">
         <v>2946.53</v>
       </c>
-      <c r="E43" s="13" t="n">
+      <c r="E43" s="16" t="n">
         <v>2620.28</v>
       </c>
+      <c r="F43" s="16" t="n">
+        <v>3941.53</v>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+      <c r="A44" s="18" t="inlineStr">
         <is>
           <t>Apr 2026</t>
         </is>
       </c>
-      <c r="B44" s="13" t="n">
+      <c r="B44" s="16" t="n">
         <v>6892.77</v>
       </c>
-      <c r="C44" s="13" t="n">
+      <c r="C44" s="16" t="n">
         <v>4189.94</v>
       </c>
-      <c r="D44" s="13" t="n">
+      <c r="D44" s="16" t="n">
         <v>2910.65</v>
       </c>
-      <c r="E44" s="13" t="n">
+      <c r="E44" s="16" t="n">
         <v>2551.07</v>
       </c>
+      <c r="F44" s="16" t="n">
+        <v>3841.97</v>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="17" t="inlineStr">
+      <c r="A45" s="18" t="inlineStr">
         <is>
           <t>May 2026</t>
         </is>
       </c>
-      <c r="B45" s="13" t="n">
+      <c r="B45" s="16" t="n">
         <v>6479.91</v>
       </c>
-      <c r="C45" s="13" t="n">
+      <c r="C45" s="16" t="n">
         <v>4029.09</v>
       </c>
-      <c r="D45" s="13" t="n">
+      <c r="D45" s="16" t="n">
         <v>2771.69</v>
       </c>
-      <c r="E45" s="13" t="n">
+      <c r="E45" s="16" t="n">
         <v>2395.19</v>
       </c>
+      <c r="F45" s="16" t="n">
+        <v>3617.64</v>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="17" t="inlineStr">
+      <c r="A46" s="18" t="inlineStr">
         <is>
           <t>Jun 2026</t>
         </is>
       </c>
-      <c r="B46" s="13" t="n">
+      <c r="B46" s="16" t="n">
         <v>6429.64</v>
       </c>
-      <c r="C46" s="13" t="n">
+      <c r="C46" s="16" t="n">
         <v>3969.45</v>
       </c>
-      <c r="D46" s="13" t="n">
+      <c r="D46" s="16" t="n">
         <v>2764.61</v>
       </c>
-      <c r="E46" s="13" t="n">
+      <c r="E46" s="16" t="n">
         <v>2383.39</v>
+      </c>
+      <c r="F46" s="16" t="n">
+        <v>3561.51</v>
       </c>
     </row>
   </sheetData>
@@ -4597,7 +5134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4605,10 +5142,11 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Bangkok STR — RevPAR by market class (monthly, This Year)</t>
         </is>
@@ -4647,803 +5185,910 @@
           <t>Upper Midscale</t>
         </is>
       </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Bangkok overall</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>Jan 2023</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="16" t="n">
         <v>4889.14</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="16" t="n">
         <v>2870.44</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="16" t="n">
         <v>1867.78</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="16" t="n">
         <v>1723.59</v>
       </c>
+      <c r="F5" s="14" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Feb 2023</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="16" t="n">
         <v>4843.13</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="16" t="n">
         <v>3172.27</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="16" t="n">
         <v>2034.2</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="16" t="n">
         <v>1795.17</v>
       </c>
+      <c r="F6" s="14" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Mar 2023</t>
         </is>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="16" t="n">
         <v>4633.91</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="16" t="n">
         <v>3295.11</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="16" t="n">
         <v>2136.46</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="16" t="n">
         <v>1811.98</v>
       </c>
+      <c r="F7" s="14" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Apr 2023</t>
         </is>
       </c>
-      <c r="B8" s="13" t="n">
+      <c r="B8" s="16" t="n">
         <v>4641.89</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="16" t="n">
         <v>3093.95</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="16" t="n">
         <v>1960.92</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="16" t="n">
         <v>1708.71</v>
       </c>
+      <c r="F8" s="14" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>May 2023</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n">
+      <c r="B9" s="16" t="n">
         <v>3823.42</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="16" t="n">
         <v>2698.86</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="16" t="n">
         <v>1864.02</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="16" t="n">
         <v>1571.84</v>
       </c>
+      <c r="F9" s="14" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Jun 2023</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n">
+      <c r="B10" s="16" t="n">
         <v>3907.12</v>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="16" t="n">
         <v>2807.79</v>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="16" t="n">
         <v>1993.01</v>
       </c>
-      <c r="E10" s="13" t="n">
+      <c r="E10" s="16" t="n">
         <v>1654.54</v>
       </c>
+      <c r="F10" s="14" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>Jul 2023</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" s="16" t="n">
         <v>4759.51</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="16" t="n">
         <v>3113.93</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="16" t="n">
         <v>2174.46</v>
       </c>
-      <c r="E11" s="13" t="n">
+      <c r="E11" s="16" t="n">
         <v>1869.38</v>
       </c>
+      <c r="F11" s="14" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Aug 2023</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n">
+      <c r="B12" s="16" t="n">
         <v>4788.02</v>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="16" t="n">
         <v>3146.79</v>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="16" t="n">
         <v>2187.14</v>
       </c>
-      <c r="E12" s="13" t="n">
+      <c r="E12" s="16" t="n">
         <v>1959.37</v>
       </c>
+      <c r="F12" s="14" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Sep 2023</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="B13" s="16" t="n">
         <v>3839.56</v>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="16" t="n">
         <v>2696.16</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="16" t="n">
         <v>1873.45</v>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E13" s="16" t="n">
         <v>1775.97</v>
       </c>
+      <c r="F13" s="14" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Oct 2023</t>
         </is>
       </c>
-      <c r="B14" s="13" t="n">
+      <c r="B14" s="16" t="n">
         <v>4103.74</v>
       </c>
-      <c r="C14" s="13" t="n">
+      <c r="C14" s="16" t="n">
         <v>2738.61</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="16" t="n">
         <v>1859.57</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="16" t="n">
         <v>1679.72</v>
       </c>
+      <c r="F14" s="14" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>Nov 2023</t>
         </is>
       </c>
-      <c r="B15" s="13" t="n">
+      <c r="B15" s="16" t="n">
         <v>4756.39</v>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C15" s="16" t="n">
         <v>3356.72</v>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="16" t="n">
         <v>2302.84</v>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E15" s="16" t="n">
         <v>2048.69</v>
       </c>
+      <c r="F15" s="14" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Dec 2023</t>
         </is>
       </c>
-      <c r="B16" s="13" t="n">
+      <c r="B16" s="16" t="n">
         <v>6058.99</v>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C16" s="16" t="n">
         <v>3884.89</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="16" t="n">
         <v>2601.8</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="16" t="n">
         <v>2309.93</v>
       </c>
+      <c r="F16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>Jan 2024</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n">
+      <c r="B17" s="16" t="n">
         <v>5277.03</v>
       </c>
-      <c r="C17" s="13" t="n">
+      <c r="C17" s="16" t="n">
         <v>3369.31</v>
       </c>
-      <c r="D17" s="13" t="n">
+      <c r="D17" s="16" t="n">
         <v>2232.68</v>
       </c>
-      <c r="E17" s="13" t="n">
+      <c r="E17" s="16" t="n">
         <v>2063.36</v>
       </c>
+      <c r="F17" s="16" t="n">
+        <v>2995.72</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Feb 2024</t>
         </is>
       </c>
-      <c r="B18" s="13" t="n">
+      <c r="B18" s="16" t="n">
         <v>6233.17</v>
       </c>
-      <c r="C18" s="13" t="n">
+      <c r="C18" s="16" t="n">
         <v>4065.68</v>
       </c>
-      <c r="D18" s="13" t="n">
+      <c r="D18" s="16" t="n">
         <v>2692.83</v>
       </c>
-      <c r="E18" s="13" t="n">
+      <c r="E18" s="16" t="n">
         <v>2299.79</v>
       </c>
+      <c r="F18" s="16" t="n">
+        <v>3508.18</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Mar 2024</t>
         </is>
       </c>
-      <c r="B19" s="13" t="n">
+      <c r="B19" s="16" t="n">
         <v>4752.28</v>
       </c>
-      <c r="C19" s="13" t="n">
+      <c r="C19" s="16" t="n">
         <v>3342.59</v>
       </c>
-      <c r="D19" s="13" t="n">
+      <c r="D19" s="16" t="n">
         <v>2267.34</v>
       </c>
-      <c r="E19" s="13" t="n">
+      <c r="E19" s="16" t="n">
         <v>1961.41</v>
       </c>
+      <c r="F19" s="16" t="n">
+        <v>2852.5</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>Apr 2024</t>
         </is>
       </c>
-      <c r="B20" s="13" t="n">
+      <c r="B20" s="16" t="n">
         <v>4747.02</v>
       </c>
-      <c r="C20" s="13" t="n">
+      <c r="C20" s="16" t="n">
         <v>3205.88</v>
       </c>
-      <c r="D20" s="13" t="n">
+      <c r="D20" s="16" t="n">
         <v>2195.46</v>
       </c>
-      <c r="E20" s="13" t="n">
+      <c r="E20" s="16" t="n">
         <v>1894.23</v>
       </c>
+      <c r="F20" s="16" t="n">
+        <v>2773.94</v>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>May 2024</t>
         </is>
       </c>
-      <c r="B21" s="13" t="n">
+      <c r="B21" s="16" t="n">
         <v>4331.31</v>
       </c>
-      <c r="C21" s="13" t="n">
+      <c r="C21" s="16" t="n">
         <v>3043.06</v>
       </c>
-      <c r="D21" s="13" t="n">
+      <c r="D21" s="16" t="n">
         <v>2155.33</v>
       </c>
-      <c r="E21" s="13" t="n">
+      <c r="E21" s="16" t="n">
         <v>1846.76</v>
       </c>
+      <c r="F21" s="16" t="n">
+        <v>2623.63</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>Jun 2024</t>
         </is>
       </c>
-      <c r="B22" s="13" t="n">
+      <c r="B22" s="16" t="n">
         <v>4642.41</v>
       </c>
-      <c r="C22" s="13" t="n">
+      <c r="C22" s="16" t="n">
         <v>3224.39</v>
       </c>
-      <c r="D22" s="13" t="n">
+      <c r="D22" s="16" t="n">
         <v>2286.24</v>
       </c>
-      <c r="E22" s="13" t="n">
+      <c r="E22" s="16" t="n">
         <v>1967.98</v>
       </c>
+      <c r="F22" s="16" t="n">
+        <v>2798.99</v>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>Jul 2024</t>
         </is>
       </c>
-      <c r="B23" s="13" t="n">
+      <c r="B23" s="16" t="n">
         <v>5155.24</v>
       </c>
-      <c r="C23" s="13" t="n">
+      <c r="C23" s="16" t="n">
         <v>3480.66</v>
       </c>
-      <c r="D23" s="13" t="n">
+      <c r="D23" s="16" t="n">
         <v>2528.93</v>
       </c>
-      <c r="E23" s="13" t="n">
+      <c r="E23" s="16" t="n">
         <v>2234.2</v>
       </c>
+      <c r="F23" s="16" t="n">
+        <v>3102.28</v>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>Aug 2024</t>
         </is>
       </c>
-      <c r="B24" s="13" t="n">
+      <c r="B24" s="16" t="n">
         <v>5514.56</v>
       </c>
-      <c r="C24" s="13" t="n">
+      <c r="C24" s="16" t="n">
         <v>3547.08</v>
       </c>
-      <c r="D24" s="13" t="n">
+      <c r="D24" s="16" t="n">
         <v>2640.82</v>
       </c>
-      <c r="E24" s="13" t="n">
+      <c r="E24" s="16" t="n">
         <v>2364.36</v>
       </c>
+      <c r="F24" s="16" t="n">
+        <v>3259.45</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>Sep 2024</t>
         </is>
       </c>
-      <c r="B25" s="13" t="n">
+      <c r="B25" s="16" t="n">
         <v>3970.65</v>
       </c>
-      <c r="C25" s="13" t="n">
+      <c r="C25" s="16" t="n">
         <v>2707.08</v>
       </c>
-      <c r="D25" s="13" t="n">
+      <c r="D25" s="16" t="n">
         <v>2050.6</v>
       </c>
-      <c r="E25" s="13" t="n">
+      <c r="E25" s="16" t="n">
         <v>1923.85</v>
       </c>
+      <c r="F25" s="16" t="n">
+        <v>2459.52</v>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>Oct 2024</t>
         </is>
       </c>
-      <c r="B26" s="13" t="n">
+      <c r="B26" s="16" t="n">
         <v>4211.24</v>
       </c>
-      <c r="C26" s="13" t="n">
+      <c r="C26" s="16" t="n">
         <v>2732.12</v>
       </c>
-      <c r="D26" s="13" t="n">
+      <c r="D26" s="16" t="n">
         <v>2075.93</v>
       </c>
-      <c r="E26" s="13" t="n">
+      <c r="E26" s="16" t="n">
         <v>1937.2</v>
       </c>
+      <c r="F26" s="16" t="n">
+        <v>2536.32</v>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="inlineStr">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>Nov 2024</t>
         </is>
       </c>
-      <c r="B27" s="13" t="n">
+      <c r="B27" s="16" t="n">
         <v>5838.23</v>
       </c>
-      <c r="C27" s="13" t="n">
+      <c r="C27" s="16" t="n">
         <v>3985.87</v>
       </c>
-      <c r="D27" s="13" t="n">
+      <c r="D27" s="16" t="n">
         <v>2896.45</v>
       </c>
-      <c r="E27" s="13" t="n">
+      <c r="E27" s="16" t="n">
         <v>2603.43</v>
       </c>
+      <c r="F27" s="16" t="n">
+        <v>3561.4</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="inlineStr">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>Dec 2024</t>
         </is>
       </c>
-      <c r="B28" s="13" t="n">
+      <c r="B28" s="16" t="n">
         <v>6932.38</v>
       </c>
-      <c r="C28" s="13" t="n">
+      <c r="C28" s="16" t="n">
         <v>4194.06</v>
       </c>
-      <c r="D28" s="13" t="n">
+      <c r="D28" s="16" t="n">
         <v>3062.61</v>
       </c>
-      <c r="E28" s="13" t="n">
+      <c r="E28" s="16" t="n">
         <v>2846.29</v>
       </c>
+      <c r="F28" s="16" t="n">
+        <v>3947.81</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="inlineStr">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>Jan 2025</t>
         </is>
       </c>
-      <c r="B29" s="13" t="n">
+      <c r="B29" s="16" t="n">
         <v>6274.09</v>
       </c>
-      <c r="C29" s="13" t="n">
+      <c r="C29" s="16" t="n">
         <v>3775.58</v>
       </c>
-      <c r="D29" s="13" t="n">
+      <c r="D29" s="16" t="n">
         <v>2743.97</v>
       </c>
-      <c r="E29" s="13" t="n">
+      <c r="E29" s="16" t="n">
         <v>2602.94</v>
       </c>
+      <c r="F29" s="16" t="n">
+        <v>3569.98</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="inlineStr">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>Feb 2025</t>
         </is>
       </c>
-      <c r="B30" s="13" t="n">
+      <c r="B30" s="16" t="n">
         <v>5657.15</v>
       </c>
-      <c r="C30" s="13" t="n">
+      <c r="C30" s="16" t="n">
         <v>3718.79</v>
       </c>
-      <c r="D30" s="13" t="n">
+      <c r="D30" s="16" t="n">
         <v>2654.53</v>
       </c>
-      <c r="E30" s="13" t="n">
+      <c r="E30" s="16" t="n">
         <v>2521.24</v>
       </c>
+      <c r="F30" s="16" t="n">
+        <v>3370.82</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="inlineStr">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>Mar 2025</t>
         </is>
       </c>
-      <c r="B31" s="13" t="n">
+      <c r="B31" s="16" t="n">
         <v>4351.17</v>
       </c>
-      <c r="C31" s="13" t="n">
+      <c r="C31" s="16" t="n">
         <v>2998.46</v>
       </c>
-      <c r="D31" s="13" t="n">
+      <c r="D31" s="16" t="n">
         <v>2171.42</v>
       </c>
-      <c r="E31" s="13" t="n">
+      <c r="E31" s="16" t="n">
         <v>2082.18</v>
       </c>
+      <c r="F31" s="16" t="n">
+        <v>2677.46</v>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="17" t="inlineStr">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>Apr 2025</t>
         </is>
       </c>
-      <c r="B32" s="13" t="n">
+      <c r="B32" s="16" t="n">
         <v>3927.1</v>
       </c>
-      <c r="C32" s="13" t="n">
+      <c r="C32" s="16" t="n">
         <v>2628.2</v>
       </c>
-      <c r="D32" s="13" t="n">
+      <c r="D32" s="16" t="n">
         <v>2018.32</v>
       </c>
-      <c r="E32" s="13" t="n">
+      <c r="E32" s="16" t="n">
         <v>1832.02</v>
       </c>
+      <c r="F32" s="16" t="n">
+        <v>2409.86</v>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>May 2025</t>
         </is>
       </c>
-      <c r="B33" s="13" t="n">
+      <c r="B33" s="16" t="n">
         <v>3645.65</v>
       </c>
-      <c r="C33" s="13" t="n">
+      <c r="C33" s="16" t="n">
         <v>2586.18</v>
       </c>
-      <c r="D33" s="13" t="n">
+      <c r="D33" s="16" t="n">
         <v>1941.86</v>
       </c>
-      <c r="E33" s="13" t="n">
+      <c r="E33" s="16" t="n">
         <v>1810.72</v>
       </c>
+      <c r="F33" s="16" t="n">
+        <v>2302.24</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="inlineStr">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>Jun 2025</t>
         </is>
       </c>
-      <c r="B34" s="13" t="n">
+      <c r="B34" s="16" t="n">
         <v>3558.1</v>
       </c>
-      <c r="C34" s="13" t="n">
+      <c r="C34" s="16" t="n">
         <v>2566.63</v>
       </c>
-      <c r="D34" s="13" t="n">
+      <c r="D34" s="16" t="n">
         <v>1978.07</v>
       </c>
-      <c r="E34" s="13" t="n">
+      <c r="E34" s="16" t="n">
         <v>1805.77</v>
       </c>
+      <c r="F34" s="16" t="n">
+        <v>2273.57</v>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="17" t="inlineStr">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>Jul 2025</t>
         </is>
       </c>
-      <c r="B35" s="13" t="n">
+      <c r="B35" s="16" t="n">
         <v>4369.3</v>
       </c>
-      <c r="C35" s="13" t="n">
+      <c r="C35" s="16" t="n">
         <v>2818.73</v>
       </c>
-      <c r="D35" s="13" t="n">
+      <c r="D35" s="16" t="n">
         <v>2212.31</v>
       </c>
-      <c r="E35" s="13" t="n">
+      <c r="E35" s="16" t="n">
         <v>2076.59</v>
       </c>
+      <c r="F35" s="16" t="n">
+        <v>2627.84</v>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="17" t="inlineStr">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>Aug 2025</t>
         </is>
       </c>
-      <c r="B36" s="13" t="n">
+      <c r="B36" s="16" t="n">
         <v>4669.24</v>
       </c>
-      <c r="C36" s="13" t="n">
+      <c r="C36" s="16" t="n">
         <v>2957</v>
       </c>
-      <c r="D36" s="13" t="n">
+      <c r="D36" s="16" t="n">
         <v>2334.22</v>
       </c>
-      <c r="E36" s="13" t="n">
+      <c r="E36" s="16" t="n">
         <v>2181.62</v>
       </c>
+      <c r="F36" s="16" t="n">
+        <v>2778.96</v>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="inlineStr">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>Sep 2025</t>
         </is>
       </c>
-      <c r="B37" s="13" t="n">
+      <c r="B37" s="16" t="n">
         <v>3401.01</v>
       </c>
-      <c r="C37" s="13" t="n">
+      <c r="C37" s="16" t="n">
         <v>2466.51</v>
       </c>
-      <c r="D37" s="13" t="n">
+      <c r="D37" s="16" t="n">
         <v>1952.57</v>
       </c>
-      <c r="E37" s="13" t="n">
+      <c r="E37" s="16" t="n">
         <v>1771.54</v>
       </c>
+      <c r="F37" s="16" t="n">
+        <v>2198.99</v>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="inlineStr">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
       </c>
-      <c r="B38" s="13" t="n">
+      <c r="B38" s="16" t="n">
         <v>4376.68</v>
       </c>
-      <c r="C38" s="13" t="n">
+      <c r="C38" s="16" t="n">
         <v>2731.84</v>
       </c>
-      <c r="D38" s="13" t="n">
+      <c r="D38" s="16" t="n">
         <v>2062.97</v>
       </c>
-      <c r="E38" s="13" t="n">
+      <c r="E38" s="16" t="n">
         <v>1952.5</v>
       </c>
+      <c r="F38" s="16" t="n">
+        <v>2548.36</v>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="17" t="inlineStr">
+      <c r="A39" s="18" t="inlineStr">
         <is>
           <t>Nov 2025</t>
         </is>
       </c>
-      <c r="B39" s="13" t="n">
+      <c r="B39" s="16" t="n">
         <v>5368.75</v>
       </c>
-      <c r="C39" s="13" t="n">
+      <c r="C39" s="16" t="n">
         <v>3525.9</v>
       </c>
-      <c r="D39" s="13" t="n">
+      <c r="D39" s="16" t="n">
         <v>2631.02</v>
       </c>
-      <c r="E39" s="13" t="n">
+      <c r="E39" s="16" t="n">
         <v>2393.99</v>
       </c>
+      <c r="F39" s="16" t="n">
+        <v>3197.15</v>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="17" t="inlineStr">
+      <c r="A40" s="18" t="inlineStr">
         <is>
           <t>Dec 2025</t>
         </is>
       </c>
-      <c r="B40" s="13" t="n">
+      <c r="B40" s="16" t="n">
         <v>6669.43</v>
       </c>
-      <c r="C40" s="13" t="n">
+      <c r="C40" s="16" t="n">
         <v>3942.16</v>
       </c>
-      <c r="D40" s="13" t="n">
+      <c r="D40" s="16" t="n">
         <v>2893.85</v>
       </c>
-      <c r="E40" s="13" t="n">
+      <c r="E40" s="16" t="n">
         <v>2616.97</v>
       </c>
+      <c r="F40" s="16" t="n">
+        <v>3739.05</v>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="17" t="inlineStr">
+      <c r="A41" s="18" t="inlineStr">
         <is>
           <t>Jan 2026</t>
         </is>
       </c>
-      <c r="B41" s="13" t="n">
+      <c r="B41" s="16" t="n">
         <v>5689.43</v>
       </c>
-      <c r="C41" s="13" t="n">
+      <c r="C41" s="16" t="n">
         <v>3363.32</v>
       </c>
-      <c r="D41" s="13" t="n">
+      <c r="D41" s="16" t="n">
         <v>2606.6</v>
       </c>
-      <c r="E41" s="13" t="n">
+      <c r="E41" s="16" t="n">
         <v>2333.65</v>
       </c>
+      <c r="F41" s="16" t="n">
+        <v>3239.27</v>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="17" t="inlineStr">
+      <c r="A42" s="18" t="inlineStr">
         <is>
           <t>Feb 2026</t>
         </is>
       </c>
-      <c r="B42" s="13" t="n">
+      <c r="B42" s="16" t="n">
         <v>6116.09</v>
       </c>
-      <c r="C42" s="13" t="n">
+      <c r="C42" s="16" t="n">
         <v>3714.6</v>
       </c>
-      <c r="D42" s="13" t="n">
+      <c r="D42" s="16" t="n">
         <v>2771.9</v>
       </c>
-      <c r="E42" s="13" t="n">
+      <c r="E42" s="16" t="n">
         <v>2501.14</v>
       </c>
+      <c r="F42" s="16" t="n">
+        <v>3516.46</v>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="inlineStr">
+      <c r="A43" s="18" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="B43" s="13" t="n">
+      <c r="B43" s="16" t="n">
         <v>4921.2</v>
       </c>
-      <c r="C43" s="13" t="n">
+      <c r="C43" s="16" t="n">
         <v>3094.43</v>
       </c>
-      <c r="D43" s="13" t="n">
+      <c r="D43" s="16" t="n">
         <v>2288.67</v>
       </c>
-      <c r="E43" s="13" t="n">
+      <c r="E43" s="16" t="n">
         <v>2091.09</v>
       </c>
+      <c r="F43" s="16" t="n">
+        <v>2887.33</v>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+      <c r="A44" s="18" t="inlineStr">
         <is>
           <t>Apr 2026</t>
         </is>
       </c>
-      <c r="B44" s="13" t="n">
+      <c r="B44" s="16" t="n">
         <v>4153.47</v>
       </c>
-      <c r="C44" s="13" t="n">
+      <c r="C44" s="16" t="n">
         <v>2660.96</v>
       </c>
-      <c r="D44" s="13" t="n">
+      <c r="D44" s="16" t="n">
         <v>2025.91</v>
       </c>
-      <c r="E44" s="13" t="n">
+      <c r="E44" s="16" t="n">
         <v>1795.38</v>
       </c>
+      <c r="F44" s="16" t="n">
+        <v>2484.6</v>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="17" t="inlineStr">
+      <c r="A45" s="18" t="inlineStr">
         <is>
           <t>May 2026</t>
         </is>
       </c>
-      <c r="B45" s="13" t="n">
+      <c r="B45" s="16" t="n">
         <v>3895.89</v>
       </c>
-      <c r="C45" s="13" t="n">
+      <c r="C45" s="16" t="n">
         <v>2561.07</v>
       </c>
-      <c r="D45" s="13" t="n">
+      <c r="D45" s="16" t="n">
         <v>1945.84</v>
       </c>
-      <c r="E45" s="13" t="n">
+      <c r="E45" s="16" t="n">
         <v>1720.68</v>
       </c>
+      <c r="F45" s="16" t="n">
+        <v>2364.44</v>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="17" t="inlineStr">
+      <c r="A46" s="18" t="inlineStr">
         <is>
           <t>Jun 2026</t>
         </is>
       </c>
-      <c r="B46" s="13" t="n">
+      <c r="B46" s="16" t="n">
         <v>3680.18</v>
       </c>
-      <c r="C46" s="13" t="n">
+      <c r="C46" s="16" t="n">
         <v>2442.69</v>
       </c>
-      <c r="D46" s="13" t="n">
+      <c r="D46" s="16" t="n">
         <v>1928.25</v>
       </c>
-      <c r="E46" s="13" t="n">
+      <c r="E46" s="16" t="n">
         <v>1732.95</v>
+      </c>
+      <c r="F46" s="16" t="n">
+        <v>2274.62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>